<commit_message>
Ref : Ref source directory
</commit_message>
<xml_diff>
--- a/docs/testing/_4.1 ManualTestV1.xlsx
+++ b/docs/testing/_4.1 ManualTestV1.xlsx
@@ -1,45 +1,21 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="FunctionList" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Test scenario" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Xác thực nhân viên" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cổng thông tin bệnh nhân" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Quy trình khám bệnh" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Phòng Ban" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Nhân sự" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Bác sĩ" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mô hình AI" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Dữ liệu đã xóa" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Audit và Blockchain" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Thông báo" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Thông tin cá nhân" sheetId="13" state="visible" r:id="rId13"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FunctionList'!$A$1:$G$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test scenario'!$A$1:$I$139</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Xác thực nhân viên'!$A$1:$H$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cổng thông tin bệnh nhân'!$A$1:$H$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Quy trình khám bệnh'!$A$1:$I$267</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Phòng Ban'!$A$1:$J$199</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Nhân sự'!$A$1:$H$109</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Bác sĩ'!$A$1:$H$112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Mô hình AI'!$A$1:$H$79</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Dữ liệu đã xóa'!$A$1:$H$109</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Audit và Blockchain'!$A$1:$H$127</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Thông báo'!$A$1:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Thông tin cá nhân'!$A$1:$H$10</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-08T09:23:00Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-11T15:10:32Z</dcterms:modified>
+  <cp:revision>7</cp:revision>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="7">
@@ -405,7 +381,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
@@ -600,7 +576,47 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="FunctionList" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Test scenario" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Xác thực nhân viên" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cổng thông tin bệnh nhân" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Quy trình khám bệnh" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Phòng Ban" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Nhân sự" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Bác sĩ" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Mô hình AI" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Dữ liệu đã xóa" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Audit và Blockchain" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Thông báo" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Thông tin cá nhân" sheetId="13" state="visible" r:id="rId13"/>
+  </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FunctionList'!$A$1:$G$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test scenario'!$A$1:$I$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Xác thực nhân viên'!$A$1:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cổng thông tin bệnh nhân'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Quy trình khám bệnh'!$A$1:$I$267</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Phòng Ban'!$A$1:$J$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Nhân sự'!$A$1:$H$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Bác sĩ'!$A$1:$H$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Mô hình AI'!$A$1:$H$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Dữ liệu đã xóa'!$A$1:$H$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Audit và Blockchain'!$A$1:$K$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Thông báo'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Thông tin cá nhân'!$A$1:$H$10</definedName>
+  </definedNames>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
@@ -1472,7 +1488,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -4166,3112 +4182,954 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl\worksheets\sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K127"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="5"/>
-    <col width="58" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="58" customWidth="1" min="8" max="8"/>
-    <col width="58" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
+    <col min="5" max="5" width="52" customWidth="1"/>
+    <col min="6" max="6" width="64" customWidth="1"/>
+    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="8" max="8" width="62" customWidth="1"/>
+    <col min="9" max="9" width="50" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Test Scenario #</t>
+          <t xml:space="preserve">Test Scenario #</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Scenario Description</t>
+          <t xml:space="preserve">Scenario Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Test Case #</t>
+          <t xml:space="preserve">Test Case #</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Test Case Description</t>
+          <t xml:space="preserve">Test Case Description</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Pre-condition</t>
+          <t xml:space="preserve">Pre-condition</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Steps</t>
+          <t xml:space="preserve">Steps</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Data Test Example</t>
+          <t xml:space="preserve">Data Test Example</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Expected Result</t>
+          <t xml:space="preserve">Expected Result</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Actual Result</t>
+          <t xml:space="preserve">Actual Result</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Pass/Failed</t>
+          <t xml:space="preserve">Pass/Failed</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="38" customHeight="1">
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="124" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S-AUD-1</t>
+          <t xml:space="preserve">KB-KT-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Xem nhật ký hệ thống</t>
+          <t xml:space="preserve">Xem audit logs và kiểm tra che dữ liệu nhạy cảm</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>TC-AUD-001</t>
+          <t xml:space="preserve">CKT-001</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Chỉ Admin được mở trang nhật ký hệ thống</t>
+          <t xml:space="preserve">Admin xem danh sách audit logs không cần quét mặt lại</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản Lễ tân đã đăng nhập và xác thực</t>
+          <t xml:space="preserve">Admin đã đăng nhập thành công; hệ thống đã có ít nhất một audit log của thao tác lưu trữ</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1. Nhập trực tiếp địa chỉ trang nhật ký</t>
+          <t xml:space="preserve">Bước 1: Tại menu quản trị, mở màn hình Audit và Blockchain.
+Bước 2: Quan sát danh sách audit logs hiển thị trên màn hình.
+Bước 3: Mở chi tiết một audit log bất kỳ.
+Bước 4: Kiểm tra hệ thống có yêu cầu quét mặt lại hay không.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Vai trò RECEPTIONIST; /admin/audit</t>
+          <t xml:space="preserve">Tài khoản: Admin; audit log mẫu là thao tác cập nhật bệnh nhân BN-KT-001 lúc 10:00</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống không hiển thị nhật ký và chuyển người dùng về trang Lễ tân. Người không có quyền không xem được người thao tác, thời gian hoặc thay đổi dữ liệu.</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="38" customHeight="1">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
+          <t xml:space="preserve">Admin xem được danh sách và chi tiết audit logs bằng session hiện tại. Hệ thống không yêu cầu quét mặt lại khi chỉ xem audit logs.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Chức năng xem audit logs hoạt động bằng session Admin hiện tại và không yêu cầu face step-up.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="124" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB-KT-01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Xem audit logs và kiểm tra che dữ liệu nhạy cảm</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CKT-002</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Người không phải Admin không được xem audit logs quản trị</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có tài khoản nhân sự không phải Admin đã đăng nhập và xác thực hợp lệ</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2. Quan sát kết quả</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="38" customHeight="1">
+          <t xml:space="preserve">Bước 1: Đăng nhập bằng tài khoản bác sĩ hoặc lễ tân.
+Bước 2: Truy cập màn hình Audit và Blockchain từ đường dẫn hoặc menu nếu có.
+Bước 3: Quan sát phản hồi của hệ thống.
+Bước 4: Kiểm tra người dùng có nhìn thấy actor, entity, hash, proof hoặc nội dung audit log hay không.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tài khoản: Doctor hoặc Receptionist; màn hình: Audit và Blockchain</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hệ thống từ chối truy cập hoặc điều hướng về khu vực đúng vai trò. Người dùng không thấy danh sách audit logs, hash, proof hoặc lịch sử thao tác quản trị.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Người không đủ quyền không xem được audit logs quản trị.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="124" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S-AUD-2</t>
+          <t xml:space="preserve">KB-KT-01</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra tính toàn vẹn</t>
+          <t xml:space="preserve">Xem audit logs và kiểm tra che dữ liệu nhạy cảm</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>TC-AUD-002</t>
+          <t xml:space="preserve">CKT-003</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Hiển thị cảnh báo khi chuỗi nhật ký không còn khớp</t>
+          <t xml:space="preserve">Audit log không hiển thị plaintext bệnh án, PII nhạy cảm, ciphertext, key hoặc artifact IPFS</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Admin đã đăng nhập; môi trường kiểm thử có bản ghi được đánh dấu không khớp</t>
+          <t xml:space="preserve">Có audit log liên quan bệnh nhân, chẩn đoán hoặc kết luận khám</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1. Mở trang Nhật ký hệ thống</t>
+          <t xml:space="preserve">Bước 1: Admin mở chi tiết audit log liên quan bệnh nhân.
+Bước 2: Kiểm tra phần thông tin thay đổi và fieldsChanged.
+Bước 3: Tìm các thông tin nhạy cảm như căn cước công dân, số điện thoại, chẩn đoán, toa thuốc, file y tế, ciphertext, key mã hóa hoặc artifact IPFS.
+Bước 4: Đối chiếu với quy định redaction đã chốt.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Một audit log kiểm thử có hash không khớp</t>
+          <t xml:space="preserve">Audit log mẫu là MedicalConclusion hoặc Patient update có trường nhạy cảm</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Giao diện hiển thị trạng thái kiểm tra thất bại, chỉ rõ bản ghi hoặc phạm vi có vấn đề và không tự sửa/xóa nhật ký. Admin có thể dùng thông tin này để điều tra.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
+          <t xml:space="preserve">Màn hình chỉ hiển thị metadata, actor, action, entity, thời điểm, batch, trạng thái kiểm chứng và fieldsChanged đã redaction. Không hiển thị plaintext bệnh án, PII nhạy cảm, ciphertext, key hoặc artifact IPFS.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Dữ liệu nhạy cảm bị redaction; màn hình không trả plaintext, ciphertext, key hoặc artifact IPFS cho người dùng.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="124" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB-KT-02</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi nhận audit logs theo nghiệp vụ lưu trữ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CKT-004</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thao tác lưu trữ thông thường tạo audit log Tier B ở trạng thái pending</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin hoặc nhân sự có quyền đã đăng nhập; có entity hợp lệ để cập nhật</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2. Chạy kiểm tra toàn vẹn</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
+          <t xml:space="preserve">Bước 1: Thực hiện một thao tác lưu trữ thông thường, ví dụ cập nhật mô tả phòng ban hoặc cập nhật thông tin không nhạy cảm của bệnh nhân.
+Bước 2: Mở màn hình Audit và Blockchain.
+Bước 3: Lọc theo entity vừa thao tác hoặc theo thời gian thao tác.
+Bước 4: Kiểm tra trạng thái batch hoặc trạng thái on-chain của audit log vừa tạo.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entity: Department PB-KT-001; thao tác: cập nhật mô tả phòng ban</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hệ thống tạo một audit log mới với actor, action, entity, entityId, thời điểm và fieldsChanged. Vì là Tier B, audit log có thể ở trạng thái pending trước khi được gom batch để anchor lên blockchain.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Audit log Tier B được tạo và giữ trạng thái pending trước khi quy trình gom batch chạy.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="124" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB-KT-02</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi nhận audit logs theo nghiệp vụ lưu trữ</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CKT-005</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thao tác quan trọng tạo audit log Tier A và được anchor ngay</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có lượt khám hợp lệ; bác sĩ phụ trách đã đăng nhập; các chỉ định bắt buộc đã xử lý hợp lệ</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>3. Mở chi tiết bản ghi lỗi</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="38" customHeight="1">
+          <t xml:space="preserve">Bước 1: Bác sĩ mở lượt khám đang phụ trách.
+Bước 2: Nhập kết luận cuối và hoàn tất lượt khám.
+Bước 3: Admin mở màn hình Audit và Blockchain.
+Bước 4: Lọc theo MedicalConclusion hoặc Visit liên quan.
+Bước 5: Kiểm tra audit log có được đưa vào quy trình anchor ngay hay không.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visit: LK-KT-001; action: tạo hoặc cập nhật kết luận cuối</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Audit log kết luận cuối được xếp Tier A. Hệ thống đóng batch cho toàn bộ audit logs đang pending theo đúng thứ tự và bắt đầu quy trình tạo checkpoint.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Audit log quan trọng được xử lý theo Tier A và không chờ lịch gom batch thông thường.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="124" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>S-AUD-3</t>
+          <t xml:space="preserve">KB-KT-03</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Bằng chứng blockchain</t>
+          <t xml:space="preserve">Kiểm chứng bằng blockchain proof</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TC-AUD-003</t>
+          <t xml:space="preserve">CKT-006</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Xác minh bằng chứng Merkle hợp lệ</t>
+          <t xml:space="preserve">Batch đã anchor hiển thị merkle root, trạng thái xác nhận và proof hợp lệ</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Một batch đã được xác nhận trên blockchain và có proof tương ứng</t>
+          <t xml:space="preserve">Có batch audit đã được anchor thành công lên blockchain trong môi trường kiểm thử</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1. Mở chi tiết audit log thuộc batch</t>
+          <t xml:space="preserve">Bước 1: Admin mở màn hình Audit và Blockchain.
+Bước 2: Chọn một audit log thuộc batch đã anchor.
+Bước 3: Mở phần kiểm chứng proof của audit log.
+Bước 4: So sánh trạng thái batch, merkle root, leaf count và thời điểm anchor.
+Bước 5: Thực hiện thao tác xác minh proof nếu màn hình có hỗ trợ.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Audit sequence thuộc batch đã anchor</t>
+          <t xml:space="preserve">Một audit log thuộc batch đã anchor thành công</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống xác nhận bằng chứng hợp lệ khi entry hash tạo lại đúng root đã lưu trên blockchain; hiển thị batch/root và trạng thái xác minh để người dùng đối chiếu.</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
+          <t xml:space="preserve">Hệ thống hiển thị batch, merkle root và trạng thái xác nhận. Proof của audit log hợp lệ và khớp với root đã lưu trên blockchain.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Batch đã anchor được xác minh bằng proof hợp lệ.</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs và blockchain</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="124" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB-KT-03</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kiểm chứng bằng blockchain proof</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CKT-007</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proof hoặc nội dung audit log bị thay đổi phải bị phát hiện là không hợp lệ</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Môi trường kiểm thử có dữ liệu giả lập proof hoặc audit log bị chỉnh sửa</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2. Chọn xem bằng chứng</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
-      <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
+          <t xml:space="preserve">Bước 1: Chuẩn bị một audit log đã anchor và một bản proof hoặc nội dung audit log đã bị sửa trong môi trường kiểm thử.
+Bước 2: Admin chạy chức năng kiểm tra tính toàn vẹn.
+Bước 3: Mở chi tiết audit log hoặc batch bị cảnh báo.
+Bước 4: Quan sát trạng thái kiểm chứng và thông báo lỗi.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proof có một sibling hash sai hoặc entryHash không còn khớp</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hệ thống không xác nhận proof hoặc audit log bị sửa là hợp lệ. Màn hình hiển thị trạng thái kiểm chứng thất bại và không tự sửa dữ liệu nếu chưa có thao tác recovery hợp lệ.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Proof hoặc audit log bị sửa bị phát hiện và không được đánh dấu hợp lệ.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs và blockchain</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="124" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB-KT-04</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phát hiện entity bị sửa trái phép và phục hồi từng bản ghi</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CKT-008</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entity bị sửa nhưng audit log mới nhất vẫn chưa anchor thì hệ thống chỉ cảnh báo, chưa cho recovery tự động</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có bản ghi bệnh nhân đã thay đổi hợp lệ; audit log tương ứng vẫn đang pending và chưa anchor lên blockchain</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>3. Thực hiện xác minh</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="38" customHeight="1">
+          <t xml:space="preserve">Bước 1: Giả lập dữ liệu bệnh nhân bị sửa trực tiếp trong database trước khi batch audit được anchor.
+Bước 2: Admin mở màn hình cảnh báo toàn vẹn dữ liệu hoặc Audit và Blockchain.
+Bước 3: Chọn entity Patient bị cảnh báo.
+Bước 4: Kiểm tra hệ thống có cho recovery từ audit log đang pending hay không.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patient BN-KT-001; dữ liệu bị sửa là họ tên và số điện thoại</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hệ thống cảnh báo entity bị lệch nhưng không cho recovery từ audit log chưa được blockchain xác nhận. Màn hình hiển thị rõ bản ghi cần kiểm tra nhưng chưa cho khôi phục tự động.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Hệ thống chặn recovery từ audit log chưa anchor.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs; bảo vệ trường hợp audit log chưa đủ tin cậy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="124" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>S-AUD-3</t>
+          <t xml:space="preserve">KB-KT-04</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Bằng chứng blockchain</t>
+          <t xml:space="preserve">Phát hiện entity bị sửa trái phép và phục hồi từng bản ghi</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>TC-AUD-004</t>
+          <t xml:space="preserve">CKT-009</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện bằng chứng Merkle bị thay đổi</t>
+          <t xml:space="preserve">Entity bị sửa sau khi batch audit đã anchor được recovery đúng bản ghi được chọn</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Có proof hợp lệ và một bản sao proof đã bị thay đổi trong môi trường test</t>
+          <t xml:space="preserve">Có Patient đã được cập nhật hợp lệ và batch audit của thay đổi đó đã anchor; sau đó dữ liệu Patient bị giả lập sửa trái phép</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1. Thay một phần tử proof bằng giá trị khác</t>
+          <t xml:space="preserve">Bước 1: Admin mở danh sách cảnh báo toàn vẹn dữ liệu.
+Bước 2: Chọn đúng Patient bị cảnh báo.
+Bước 3: Xem metadata được phép xem, không xem dữ liệu nhạy cảm.
+Bước 4: Nhập lý do recovery.
+Bước 5: Xác nhận recovery đúng entity được chọn.
+Bước 6: Kiểm tra lại chi tiết Patient và audit log phục hồi.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Proof có một sibling hash sai</t>
+          <t xml:space="preserve">Patient BN-KT-001; trạng thái cảnh báo: bị chỉnh sửa trái phép; lý do: khôi phục dữ liệu bị chỉnh sửa trái phép</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Kết quả xác minh là không hợp lệ. Hệ thống không báo dữ liệu toàn vẹn và không thay đổi audit log hoặc root đã lưu.</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-    </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+          <t xml:space="preserve">Hệ thống lấy trusted snapshot mới nhất đã được blockchain xác nhận, recovery đúng Patient được chọn, không phục hồi lan sang entity khác. Sau recovery, entity hết cảnh báo và tạo audit log AUDIT_ENTITY_RECOVERED.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Entity recovery khôi phục đúng một Patient, không lộ dữ liệu nhạy cảm trên màn hình.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs; recovery theo từng entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="124" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB-KT-04</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phát hiện entity bị sửa trái phép và phục hồi từng bản ghi</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CKT-010</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khi audit log pending bị sửa hash, hệ thống dừng anchor lên blockchain</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có audit log pending trong hệ thống; môi trường kiểm thử có thao tác giả lập hash bị sửa</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2. Thực hiện xác minh</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-    </row>
-    <row r="12" ht="38" customHeight="1">
+          <t xml:space="preserve">Bước 1: Tạo một thao tác lưu trữ để phát sinh audit log pending.
+Bước 2: Giả lập afterHash hoặc entryHash của audit log bị thay đổi.
+Bước 3: Admin hoặc background job kích hoạt quy trình anchor audit logs.
+Bước 4: Quan sát trạng thái batch và thông báo cảnh báo.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Audit log pending bị sửa afterHash thành giá trị không khớp</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hệ thống phát hiện hash không khớp, dừng commit checkpoint lên blockchain, không tạo batch đã anchor từ dữ liệu sai và giữ cảnh báo để xử lý.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Quy trình anchor bị chặn khi nội dung audit log pending bị sửa.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs; chống anchor root sai</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="124" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>S-AUD-4</t>
+          <t xml:space="preserve">KB-KT-05</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Quyền ghi blockchain</t>
+          <t xml:space="preserve">Phục hồi lịch sử audit logs bằng encrypted IPFS artifact</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>TC-AUD-005</t>
+          <t xml:space="preserve">CKT-011</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Ví không được cấp quyền không thể ghi root audit</t>
+          <t xml:space="preserve">Audit batch bị sửa trong database được phục hồi từ encrypted IPFS artifact</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Hợp đồng lưu bằng chứng audit đã được triển khai; ví kiểm thử không nằm trong danh sách được phép ghi dữ liệu</t>
+          <t xml:space="preserve">Có audit batch đã anchor và có artifact IPFS tương ứng; sau đó một audit log trong database bị giả lập sửa entryHash</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>1. Kết nối bằng ví không được cấp quyền</t>
+          <t xml:space="preserve">Bước 1: Admin mở màn hình Audit và Blockchain.
+Bước 2: Chọn batch bị cảnh báo sai lệch.
+Bước 3: Thực hiện quy trình recovery audit batch theo quyền Admin.
+Bước 4: Hệ thống tải encrypted artifact từ IPFS đã cấu hình.
+Bước 5: Kiểm tra lại trạng thái batch và audit log sau recovery.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Mã lô mới; giá trị kiểm tra hợp lệ; ví không được cấp quyền</t>
+          <t xml:space="preserve">Batch AUD-KT-001; lỗi là entryHash trong database không khớp root trên blockchain</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Giao dịch bị từ chối. Không tạo mốc kiểm tra mới, không phát thông báo ghi thành công và lô dữ liệu vẫn chưa có bằng chứng trên blockchain.</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
-    </row>
-    <row r="13" ht="38" customHeight="1">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
+          <t xml:space="preserve">Hệ thống kiểm artifactHash, giải mã nội bộ, kiểm bundle root khớp blockchain, phục hồi các audit logs của batch và đưa audit logs về trạng thái đã anchor.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Batch recovery trả trạng thái recovered và khôi phục đúng audit log bị sửa.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs; IPFS chỉ chứa encrypted audit artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="124" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB-KT-05</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phục hồi lịch sử audit logs bằng encrypted IPFS artifact</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CKT-012</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Artifact IPFS, hash hoặc GCM tag không hợp lệ thì recovery dừng và không ghi đè database</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có batch đã anchor; môi trường kiểm thử giả lập artifact không tải được hoặc file mã hóa bị sửa</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2. Gọi chức năng commit root</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-    </row>
-    <row r="14" ht="38" customHeight="1">
+          <t xml:space="preserve">Bước 1: Admin chọn batch cần recovery.
+Bước 2: Giả lập một lỗi: không tải được artifact, artifactHash không khớp, GCM tag sai hoặc bundle root không khớp.
+Bước 3: Thực hiện recovery audit batch.
+Bước 4: Kiểm tra các audit logs và trạng thái batch sau khi lỗi xảy ra.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID sai hoặc encrypted artifact bị thay đổi</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hệ thống dừng recovery, hiển thị lỗi kiểm chứng rõ ràng, không ghi đè audit logs và không đánh dấu batch là đã recovery.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Recovery bị từ chối khi artifact, hash hoặc GCM tag không hợp lệ.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs; không trả decrypted bundle ra màn hình</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="124" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>S-AUD-5</t>
+          <t xml:space="preserve">KB-KT-06</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Bảo vệ dữ liệu y tế</t>
+          <t xml:space="preserve">Khả năng chịu lỗi khi server hoặc blockchain tạm thời không sẵn sàng</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>TC-AUD-006</t>
+          <t xml:space="preserve">CKT-013</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Blockchain không chứa thông tin bệnh nhân hoặc nội dung chẩn đoán</t>
+          <t xml:space="preserve">Server dừng hoặc restart trước khi batch được anchor thì audit log vẫn được xử lý tiếp sau khi hệ thống chạy lại</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Một bệnh án đã được kết luận và audit đã được anchor</t>
+          <t xml:space="preserve">Có audit log pending đã được ghi bền vững trong database; mô phỏng server dừng trước khi hoàn tất anchor blockchain</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>1. Mở dữ liệu transaction/event/checkpoint</t>
+          <t xml:space="preserve">Bước 1: Thực hiện một thao tác lưu trữ để tạo audit log pending.
+Bước 2: Giả lập server dừng trước khi batch được anchor.
+Bước 3: Khởi động lại hệ thống.
+Bước 4: Chờ background job của audit logs hoạt động lại hoặc kích hoạt kiểm tra batch.
+Bước 5: Mở màn hình Audit và Blockchain để kiểm tra trạng thái audit log và batch.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Bệnh án có tên, CCCD, chẩn đoán và toa thuốc</t>
+          <t xml:space="preserve">Audit log pending của Patient BN-KT-001 hoặc Department PB-KT-001</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu blockchain chỉ có hash, batch, thời gian và metadata kỹ thuật cần thiết. Không xuất hiện tên, CCCD, số điện thoại, chẩn đoán, toa thuốc hoặc file y tế.</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-    </row>
-    <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
+          <t xml:space="preserve">Sau khi restart, hệ thống tìm lại audit log pending từ database, tiếp tục quy trình tạo artifact và checkpoint, không tạo audit log trùng.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Audit log pending được xử lý tiếp sau restart, không mất log và không tạo batch trùng.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs; restart resilience</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="124" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB-KT-06</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Khả năng chịu lỗi khi server hoặc blockchain tạm thời không sẵn sàng</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CKT-014</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mất kết nối blockchain sau khi artifact đã sẵn sàng thì hệ thống retry cùng artifact, không tạo artifact khác</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có batch đã tạo artifact nhưng lần commit checkpoint đầu tiên lên blockchain bị lỗi kết nối</t>
+        </is>
+      </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2. Đối chiếu với bệnh án trong database</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
-    </row>
-    <row r="16" ht="38" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>S-AUD-6</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Ghi anchor thủ công</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>TC-AUD-007</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Không cho người không phải Admin yêu cầu anchor ngay</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Tài khoản Doctor đã đăng nhập và xác thực</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>1. Gửi yêu cầu thực hiện anchor ngay</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Vai trò DOCTOR</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Yêu cầu bị từ chối vì không đủ quyền. Không tạo batch/giao dịch mới và không làm thay đổi trạng thái các audit log đang chờ.</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
-    </row>
-    <row r="17" ht="38" customHeight="1">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>2. Kiểm tra batch và giao dịch mới</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
-    </row>
-    <row r="18" ht="38" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>S-AUD-7</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Lỗi kết nối blockchain</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>TC-AUD-008</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Không báo thành công giả khi mạng blockchain không phản hồi</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Có nhật ký đang chờ đưa bằng chứng lên blockchain; mô phỏng mất kết nối với mạng blockchain</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>1. Admin chọn đưa bằng chứng lên blockchain ngay</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Mạng blockchain không phản hồi cho đến khi hết thời gian chờ</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Giao diện thông báo chưa thể hoàn tất việc đưa bằng chứng lên blockchain. Không hiển thị trạng thái đã xác nhận khi chưa có giao dịch thành công; nhật ký trong hệ thống vẫn được giữ để thử lại.</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
-    </row>
-    <row r="19" ht="38" customHeight="1">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>2. Chờ đến khi yêu cầu hết thời gian</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
-    </row>
-    <row r="20" ht="38" customHeight="1">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>3. Tải lại danh sách batch</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
-      <c r="K20" s="5" t="n"/>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-1</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Nhân sự</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-STF-001</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>Tạo Nhân sự và xác nhận Nhật ký lưu đúng hành động</t>
-        </is>
-      </c>
-      <c r="E21" s="19" t="inlineStr">
-        <is>
-          <t>Admin đã đăng nhập; chưa có bản ghi mang mã NV-AUD-01</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý nhân sự</t>
-        </is>
-      </c>
-      <c r="G21" s="19" t="inlineStr">
-        <is>
-          <t>NV-AUD-01; dữ liệu giả hợp lệ</t>
-        </is>
-      </c>
-      <c r="H21" s="19" t="inlineStr">
-        <is>
-          <t>Bản ghi được tạo đúng một lần. Nhật ký có entity StaffProfile, action CREATE, đúng ID/mã, Admin và thời gian. Các trường được tạo xuất hiện trong danh sách thay đổi; không hiển thị mật khẩu, khóa bí mật hoặc dữ liệu nhận dạng khuôn mặt.</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="n"/>
-      <c r="J21" s="19" t="n"/>
-      <c r="K21" s="19" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="19" t="inlineStr">
-        <is>
-          <t>2. Chọn thêm nhân sự, nhập dữ liệu có mã NV-AUD-01 rồi lưu</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="n"/>
-      <c r="H22" s="4" t="n"/>
-      <c r="I22" s="4" t="n"/>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="n"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận bản ghi xuất hiện trong danh sách</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="n"/>
-      <c r="I23" s="4" t="n"/>
-      <c r="J23" s="4" t="n"/>
-      <c r="K23" s="4" t="n"/>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại thời gian hoàn tất</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="n"/>
-      <c r="I24" s="4" t="n"/>
-      <c r="J24" s="4" t="n"/>
-      <c r="K24" s="4" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
-      <c r="I25" s="4" t="n"/>
-      <c r="J25" s="4" t="n"/>
-      <c r="K25" s="4" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="4" t="n"/>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>6. Lọc theo đối tượng Nhân sự và tìm NV-AUD-01</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="n"/>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log mới nhất và đối chiếu thông tin</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="n"/>
-      <c r="K27" s="5" t="n"/>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-1</t>
-        </is>
-      </c>
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Nhân sự</t>
-        </is>
-      </c>
-      <c r="C28" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-STF-002</t>
-        </is>
-      </c>
-      <c r="D28" s="19" t="inlineStr">
-        <is>
-          <t>Sửa một trường của Nhân sự và kiểm tra giá trị trước/sau trong Nhật ký</t>
-        </is>
-      </c>
-      <c r="E28" s="19" t="inlineStr">
-        <is>
-          <t>Nhân sự NV-AUD-01 tồn tại; họ tên hiện là Nguyễn Văn Kiểm Thử</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý nhân sự và chọn NV-AUD-01</t>
-        </is>
-      </c>
-      <c r="G28" s="19" t="inlineStr">
-        <is>
-          <t>họ tên: Nguyễn Văn Kiểm Thử → Nguyễn Văn Kiểm Tra</t>
-        </is>
-      </c>
-      <c r="H28" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký có action UPDATE và chỉ ghi đúng trường họ tên đã đổi từ Nguyễn Văn Kiểm Thử sang Nguyễn Văn Kiểm Tra. Các trường không chỉnh sửa không bị ghi nhầm. Người thực hiện, thời gian và ID đối tượng đúng với thao tác vừa hoàn tất.</t>
-        </is>
-      </c>
-      <c r="I28" s="19" t="n"/>
-      <c r="J28" s="19" t="n"/>
-      <c r="K28" s="19" t="n"/>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="4" t="n"/>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="19" t="inlineStr">
-        <is>
-          <t>2. Đổi họ tên từ Nguyễn Văn Kiểm Thử thành Nguyễn Văn Kiểm Tra rồi lưu</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="n"/>
-      <c r="J29" s="4" t="n"/>
-      <c r="K29" s="4" t="n"/>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận màn hình hiển thị giá trị mới</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="n"/>
-      <c r="H30" s="4" t="n"/>
-      <c r="I30" s="4" t="n"/>
-      <c r="J30" s="4" t="n"/>
-      <c r="K30" s="4" t="n"/>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="19" t="inlineStr">
-        <is>
-          <t>4. Mở Nhật ký hệ thống và tìm {key}</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="4" t="n"/>
-      <c r="J31" s="4" t="n"/>
-      <c r="K31" s="4" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở log UPDATE mới nhất</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
-      <c r="I32" s="4" t="n"/>
-      <c r="J32" s="4" t="n"/>
-      <c r="K32" s="4" t="n"/>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="5" t="n"/>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="19" t="inlineStr">
-        <is>
-          <t>6. Đối chiếu trường thay đổi và giá trị trước/sau</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="5" t="n"/>
-      <c r="K33" s="5" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-1</t>
-        </is>
-      </c>
-      <c r="B34" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Nhân sự</t>
-        </is>
-      </c>
-      <c r="C34" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-STF-003</t>
-        </is>
-      </c>
-      <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>Ẩn rồi hiện lại Nhân sự và kiểm tra hai lần thay đổi trạng thái</t>
-        </is>
-      </c>
-      <c r="E34" s="19" t="inlineStr">
-        <is>
-          <t>Nhân sự NV-AUD-01 đang hoạt động</t>
-        </is>
-      </c>
-      <c r="F34" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý nhân sự và chọn Ẩn NV-AUD-01</t>
-        </is>
-      </c>
-      <c r="G34" s="19" t="inlineStr">
-        <is>
-          <t>NV-AUD-01; ACTIVE → INACTIVE → ACTIVE</t>
-        </is>
-      </c>
-      <c r="H34" s="19" t="inlineStr">
-        <is>
-          <t>Mỗi thao tác thành công có một log UPDATE phản ánh đúng thay đổi Trạng thái. Log ẩn ghi Đang hoạt động sang Đã ẩn; log hiện lại ghi Đã ẩn sang Đang hoạt động. Không được ghi action DELETE vì Ẩn không phải Xóa.</t>
-        </is>
-      </c>
-      <c r="I34" s="19" t="n"/>
-      <c r="J34" s="19" t="n"/>
-      <c r="K34" s="19" t="n"/>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="19" t="inlineStr">
-        <is>
-          <t>2. Kiểm tra bản ghi chuyển sang Đã ẩn</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="n"/>
-      <c r="H35" s="4" t="n"/>
-      <c r="I35" s="4" t="n"/>
-      <c r="J35" s="4" t="n"/>
-      <c r="K35" s="4" t="n"/>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="4" t="n"/>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="19" t="inlineStr">
-        <is>
-          <t>3. Mở Nhật ký và tìm log mới nhất</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="n"/>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="4" t="n"/>
-      <c r="J36" s="4" t="n"/>
-      <c r="K36" s="4" t="n"/>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="19" t="inlineStr">
-        <is>
-          <t>4. Quay lại trang quản lý và chọn Hiện</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
-      <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="n"/>
-      <c r="K37" s="4" t="n"/>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="5" t="n"/>
-      <c r="B38" s="5" t="n"/>
-      <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở Nhật ký và đối chiếu log mới nhất lần nữa</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="5" t="n"/>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="5" t="n"/>
-      <c r="K38" s="5" t="n"/>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-2</t>
-        </is>
-      </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Bác sĩ</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-DOC-001</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>Tạo Bác sĩ và xác nhận Nhật ký lưu đúng hành động</t>
-        </is>
-      </c>
-      <c r="E39" s="19" t="inlineStr">
-        <is>
-          <t>Admin đã đăng nhập; chưa có bản ghi mang mã BS-AUD-01</t>
-        </is>
-      </c>
-      <c r="F39" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý bác sĩ</t>
-        </is>
-      </c>
-      <c r="G39" s="19" t="inlineStr">
-        <is>
-          <t>BS-AUD-01; dữ liệu giả hợp lệ</t>
-        </is>
-      </c>
-      <c r="H39" s="19" t="inlineStr">
-        <is>
-          <t>Bản ghi được tạo đúng một lần. Nhật ký có entity DoctorProfile, action CREATE, đúng ID/mã, Admin và thời gian. Các trường được tạo xuất hiện trong danh sách thay đổi; không hiển thị mật khẩu, khóa bí mật hoặc dữ liệu nhận dạng khuôn mặt.</t>
-        </is>
-      </c>
-      <c r="I39" s="19" t="n"/>
-      <c r="J39" s="19" t="n"/>
-      <c r="K39" s="19" t="n"/>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="4" t="n"/>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="19" t="inlineStr">
-        <is>
-          <t>2. Chọn thêm bác sĩ, nhập dữ liệu có mã BS-AUD-01 rồi lưu</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="n"/>
-      <c r="H40" s="4" t="n"/>
-      <c r="I40" s="4" t="n"/>
-      <c r="J40" s="4" t="n"/>
-      <c r="K40" s="4" t="n"/>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="4" t="n"/>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận bản ghi xuất hiện trong danh sách</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="4" t="n"/>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại thời gian hoàn tất</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="n"/>
-      <c r="H42" s="4" t="n"/>
-      <c r="I42" s="4" t="n"/>
-      <c r="J42" s="4" t="n"/>
-      <c r="K42" s="4" t="n"/>
-    </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="4" t="n"/>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="n"/>
-      <c r="H43" s="4" t="n"/>
-      <c r="I43" s="4" t="n"/>
-      <c r="J43" s="4" t="n"/>
-      <c r="K43" s="4" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="4" t="n"/>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="19" t="inlineStr">
-        <is>
-          <t>6. Lọc theo đối tượng Bác sĩ và tìm BS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="n"/>
-      <c r="H44" s="4" t="n"/>
-      <c r="I44" s="4" t="n"/>
-      <c r="J44" s="4" t="n"/>
-      <c r="K44" s="4" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="5" t="n"/>
-      <c r="B45" s="5" t="n"/>
-      <c r="C45" s="5" t="n"/>
-      <c r="D45" s="5" t="n"/>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log mới nhất và đối chiếu thông tin</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="5" t="n"/>
-      <c r="I45" s="5" t="n"/>
-      <c r="J45" s="5" t="n"/>
-      <c r="K45" s="5" t="n"/>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-2</t>
-        </is>
-      </c>
-      <c r="B46" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Bác sĩ</t>
-        </is>
-      </c>
-      <c r="C46" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-DOC-002</t>
-        </is>
-      </c>
-      <c r="D46" s="19" t="inlineStr">
-        <is>
-          <t>Sửa một trường của Bác sĩ và kiểm tra giá trị trước/sau trong Nhật ký</t>
-        </is>
-      </c>
-      <c r="E46" s="19" t="inlineStr">
-        <is>
-          <t>Bác sĩ BS-AUD-01 tồn tại; chuyên khoa hiện là Tim mạch</t>
-        </is>
-      </c>
-      <c r="F46" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý bác sĩ và chọn BS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G46" s="19" t="inlineStr">
-        <is>
-          <t>chuyên khoa: Tim mạch → Hô hấp</t>
-        </is>
-      </c>
-      <c r="H46" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký có action UPDATE và chỉ ghi đúng trường chuyên khoa đã đổi từ Tim mạch sang Hô hấp. Các trường không chỉnh sửa không bị ghi nhầm. Người thực hiện, thời gian và ID đối tượng đúng với thao tác vừa hoàn tất.</t>
-        </is>
-      </c>
-      <c r="I46" s="19" t="n"/>
-      <c r="J46" s="19" t="n"/>
-      <c r="K46" s="19" t="n"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="19" t="inlineStr">
-        <is>
-          <t>2. Đổi chuyên khoa từ Tim mạch thành Hô hấp rồi lưu</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="n"/>
-      <c r="H47" s="4" t="n"/>
-      <c r="I47" s="4" t="n"/>
-      <c r="J47" s="4" t="n"/>
-      <c r="K47" s="4" t="n"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="4" t="n"/>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận màn hình hiển thị giá trị mới</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="n"/>
-      <c r="H48" s="4" t="n"/>
-      <c r="I48" s="4" t="n"/>
-      <c r="J48" s="4" t="n"/>
-      <c r="K48" s="4" t="n"/>
-    </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="19" t="inlineStr">
-        <is>
-          <t>4. Mở Nhật ký hệ thống và tìm {key}</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="n"/>
-      <c r="H49" s="4" t="n"/>
-      <c r="I49" s="4" t="n"/>
-      <c r="J49" s="4" t="n"/>
-      <c r="K49" s="4" t="n"/>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="4" t="n"/>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở log UPDATE mới nhất</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="n"/>
-      <c r="H50" s="4" t="n"/>
-      <c r="I50" s="4" t="n"/>
-      <c r="J50" s="4" t="n"/>
-      <c r="K50" s="4" t="n"/>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="5" t="n"/>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="19" t="inlineStr">
-        <is>
-          <t>6. Đối chiếu trường thay đổi và giá trị trước/sau</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="5" t="n"/>
-      <c r="I51" s="5" t="n"/>
-      <c r="J51" s="5" t="n"/>
-      <c r="K51" s="5" t="n"/>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-2</t>
-        </is>
-      </c>
-      <c r="B52" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Bác sĩ</t>
-        </is>
-      </c>
-      <c r="C52" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-DOC-003</t>
-        </is>
-      </c>
-      <c r="D52" s="19" t="inlineStr">
-        <is>
-          <t>Ẩn rồi hiện lại Bác sĩ và kiểm tra hai lần thay đổi trạng thái</t>
-        </is>
-      </c>
-      <c r="E52" s="19" t="inlineStr">
-        <is>
-          <t>Bác sĩ BS-AUD-01 đang hoạt động</t>
-        </is>
-      </c>
-      <c r="F52" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý bác sĩ và chọn Ẩn BS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G52" s="19" t="inlineStr">
-        <is>
-          <t>BS-AUD-01; ACTIVE → INACTIVE → ACTIVE</t>
-        </is>
-      </c>
-      <c r="H52" s="19" t="inlineStr">
-        <is>
-          <t>Mỗi thao tác thành công có một log UPDATE phản ánh đúng thay đổi Trạng thái. Log ẩn ghi Đang hoạt động sang Đã ẩn; log hiện lại ghi Đã ẩn sang Đang hoạt động. Không được ghi action DELETE vì Ẩn không phải Xóa.</t>
-        </is>
-      </c>
-      <c r="I52" s="19" t="n"/>
-      <c r="J52" s="19" t="n"/>
-      <c r="K52" s="19" t="n"/>
-    </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="4" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="19" t="inlineStr">
-        <is>
-          <t>2. Kiểm tra bản ghi chuyển sang Đã ẩn</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="n"/>
-      <c r="H53" s="4" t="n"/>
-      <c r="I53" s="4" t="n"/>
-      <c r="J53" s="4" t="n"/>
-      <c r="K53" s="4" t="n"/>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="4" t="n"/>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="19" t="inlineStr">
-        <is>
-          <t>3. Mở Nhật ký và tìm log mới nhất</t>
-        </is>
-      </c>
-      <c r="G54" s="4" t="n"/>
-      <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="n"/>
-      <c r="K54" s="4" t="n"/>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="4" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="19" t="inlineStr">
-        <is>
-          <t>4. Quay lại trang quản lý và chọn Hiện</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="n"/>
-      <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
-      <c r="K55" s="4" t="n"/>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="5" t="n"/>
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="5" t="n"/>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="5" t="n"/>
-      <c r="F56" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở Nhật ký và đối chiếu log mới nhất lần nữa</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="n"/>
-      <c r="H56" s="5" t="n"/>
-      <c r="I56" s="5" t="n"/>
-      <c r="J56" s="5" t="n"/>
-      <c r="K56" s="5" t="n"/>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-3</t>
-        </is>
-      </c>
-      <c r="B57" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Phòng ban</t>
-        </is>
-      </c>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-DEP-001</t>
-        </is>
-      </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Tạo Phòng ban và xác nhận Nhật ký lưu đúng hành động</t>
-        </is>
-      </c>
-      <c r="E57" s="19" t="inlineStr">
-        <is>
-          <t>Admin đã đăng nhập; chưa có bản ghi mang mã PB-AUD-01</t>
-        </is>
-      </c>
-      <c r="F57" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý phòng ban</t>
-        </is>
-      </c>
-      <c r="G57" s="19" t="inlineStr">
-        <is>
-          <t>PB-AUD-01; dữ liệu giả hợp lệ</t>
-        </is>
-      </c>
-      <c r="H57" s="19" t="inlineStr">
-        <is>
-          <t>Bản ghi được tạo đúng một lần. Nhật ký có entity Department, action CREATE, đúng ID/mã, Admin và thời gian. Các trường được tạo xuất hiện trong danh sách thay đổi; không hiển thị mật khẩu, khóa bí mật hoặc dữ liệu nhận dạng khuôn mặt.</t>
-        </is>
-      </c>
-      <c r="I57" s="19" t="n"/>
-      <c r="J57" s="19" t="n"/>
-      <c r="K57" s="19" t="n"/>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="4" t="n"/>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="19" t="inlineStr">
-        <is>
-          <t>2. Chọn thêm phòng ban, nhập dữ liệu có mã PB-AUD-01 rồi lưu</t>
-        </is>
-      </c>
-      <c r="G58" s="4" t="n"/>
-      <c r="H58" s="4" t="n"/>
-      <c r="I58" s="4" t="n"/>
-      <c r="J58" s="4" t="n"/>
-      <c r="K58" s="4" t="n"/>
-    </row>
-    <row r="59" ht="30" customHeight="1">
-      <c r="A59" s="4" t="n"/>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="4" t="n"/>
-      <c r="E59" s="4" t="n"/>
-      <c r="F59" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận bản ghi xuất hiện trong danh sách</t>
-        </is>
-      </c>
-      <c r="G59" s="4" t="n"/>
-      <c r="H59" s="4" t="n"/>
-      <c r="I59" s="4" t="n"/>
-      <c r="J59" s="4" t="n"/>
-      <c r="K59" s="4" t="n"/>
-    </row>
-    <row r="60" ht="30" customHeight="1">
-      <c r="A60" s="4" t="n"/>
-      <c r="B60" s="4" t="n"/>
-      <c r="C60" s="4" t="n"/>
-      <c r="D60" s="4" t="n"/>
-      <c r="E60" s="4" t="n"/>
-      <c r="F60" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại thời gian hoàn tất</t>
-        </is>
-      </c>
-      <c r="G60" s="4" t="n"/>
-      <c r="H60" s="4" t="n"/>
-      <c r="I60" s="4" t="n"/>
-      <c r="J60" s="4" t="n"/>
-      <c r="K60" s="4" t="n"/>
-    </row>
-    <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="4" t="n"/>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="4" t="n"/>
-      <c r="E61" s="4" t="n"/>
-      <c r="F61" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="n"/>
-      <c r="H61" s="4" t="n"/>
-      <c r="I61" s="4" t="n"/>
-      <c r="J61" s="4" t="n"/>
-      <c r="K61" s="4" t="n"/>
-    </row>
-    <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="4" t="n"/>
-      <c r="B62" s="4" t="n"/>
-      <c r="C62" s="4" t="n"/>
-      <c r="D62" s="4" t="n"/>
-      <c r="E62" s="4" t="n"/>
-      <c r="F62" s="19" t="inlineStr">
-        <is>
-          <t>6. Lọc theo đối tượng Phòng ban và tìm PB-AUD-01</t>
-        </is>
-      </c>
-      <c r="G62" s="4" t="n"/>
-      <c r="H62" s="4" t="n"/>
-      <c r="I62" s="4" t="n"/>
-      <c r="J62" s="4" t="n"/>
-      <c r="K62" s="4" t="n"/>
-    </row>
-    <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="5" t="n"/>
-      <c r="B63" s="5" t="n"/>
-      <c r="C63" s="5" t="n"/>
-      <c r="D63" s="5" t="n"/>
-      <c r="E63" s="5" t="n"/>
-      <c r="F63" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log mới nhất và đối chiếu thông tin</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="n"/>
-      <c r="H63" s="5" t="n"/>
-      <c r="I63" s="5" t="n"/>
-      <c r="J63" s="5" t="n"/>
-      <c r="K63" s="5" t="n"/>
-    </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-3</t>
-        </is>
-      </c>
-      <c r="B64" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Phòng ban</t>
-        </is>
-      </c>
-      <c r="C64" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-DEP-002</t>
-        </is>
-      </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>Sửa một trường của Phòng ban và kiểm tra giá trị trước/sau trong Nhật ký</t>
-        </is>
-      </c>
-      <c r="E64" s="19" t="inlineStr">
-        <is>
-          <t>Phòng ban PB-AUD-01 tồn tại; tầng hiện là 2</t>
-        </is>
-      </c>
-      <c r="F64" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý phòng ban và chọn PB-AUD-01</t>
-        </is>
-      </c>
-      <c r="G64" s="19" t="inlineStr">
-        <is>
-          <t>tầng: 2 → 3</t>
-        </is>
-      </c>
-      <c r="H64" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký có action UPDATE và chỉ ghi đúng trường tầng đã đổi từ 2 sang 3. Các trường không chỉnh sửa không bị ghi nhầm. Người thực hiện, thời gian và ID đối tượng đúng với thao tác vừa hoàn tất.</t>
-        </is>
-      </c>
-      <c r="I64" s="19" t="n"/>
-      <c r="J64" s="19" t="n"/>
-      <c r="K64" s="19" t="n"/>
-    </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="4" t="n"/>
-      <c r="B65" s="4" t="n"/>
-      <c r="C65" s="4" t="n"/>
-      <c r="D65" s="4" t="n"/>
-      <c r="E65" s="4" t="n"/>
-      <c r="F65" s="19" t="inlineStr">
-        <is>
-          <t>2. Đổi tầng từ 2 thành 3 rồi lưu</t>
-        </is>
-      </c>
-      <c r="G65" s="4" t="n"/>
-      <c r="H65" s="4" t="n"/>
-      <c r="I65" s="4" t="n"/>
-      <c r="J65" s="4" t="n"/>
-      <c r="K65" s="4" t="n"/>
-    </row>
-    <row r="66" ht="30" customHeight="1">
-      <c r="A66" s="4" t="n"/>
-      <c r="B66" s="4" t="n"/>
-      <c r="C66" s="4" t="n"/>
-      <c r="D66" s="4" t="n"/>
-      <c r="E66" s="4" t="n"/>
-      <c r="F66" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận màn hình hiển thị giá trị mới</t>
-        </is>
-      </c>
-      <c r="G66" s="4" t="n"/>
-      <c r="H66" s="4" t="n"/>
-      <c r="I66" s="4" t="n"/>
-      <c r="J66" s="4" t="n"/>
-      <c r="K66" s="4" t="n"/>
-    </row>
-    <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="4" t="n"/>
-      <c r="B67" s="4" t="n"/>
-      <c r="C67" s="4" t="n"/>
-      <c r="D67" s="4" t="n"/>
-      <c r="E67" s="4" t="n"/>
-      <c r="F67" s="19" t="inlineStr">
-        <is>
-          <t>4. Mở Nhật ký hệ thống và tìm {key}</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="n"/>
-      <c r="H67" s="4" t="n"/>
-      <c r="I67" s="4" t="n"/>
-      <c r="J67" s="4" t="n"/>
-      <c r="K67" s="4" t="n"/>
-    </row>
-    <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="4" t="n"/>
-      <c r="B68" s="4" t="n"/>
-      <c r="C68" s="4" t="n"/>
-      <c r="D68" s="4" t="n"/>
-      <c r="E68" s="4" t="n"/>
-      <c r="F68" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở log UPDATE mới nhất</t>
-        </is>
-      </c>
-      <c r="G68" s="4" t="n"/>
-      <c r="H68" s="4" t="n"/>
-      <c r="I68" s="4" t="n"/>
-      <c r="J68" s="4" t="n"/>
-      <c r="K68" s="4" t="n"/>
-    </row>
-    <row r="69" ht="30" customHeight="1">
-      <c r="A69" s="5" t="n"/>
-      <c r="B69" s="5" t="n"/>
-      <c r="C69" s="5" t="n"/>
-      <c r="D69" s="5" t="n"/>
-      <c r="E69" s="5" t="n"/>
-      <c r="F69" s="19" t="inlineStr">
-        <is>
-          <t>6. Đối chiếu trường thay đổi và giá trị trước/sau</t>
-        </is>
-      </c>
-      <c r="G69" s="5" t="n"/>
-      <c r="H69" s="5" t="n"/>
-      <c r="I69" s="5" t="n"/>
-      <c r="J69" s="5" t="n"/>
-      <c r="K69" s="5" t="n"/>
-    </row>
-    <row r="70" ht="30" customHeight="1">
-      <c r="A70" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-3</t>
-        </is>
-      </c>
-      <c r="B70" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Phòng ban</t>
-        </is>
-      </c>
-      <c r="C70" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-DEP-003</t>
-        </is>
-      </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>Ẩn rồi hiện lại Phòng ban và kiểm tra hai lần thay đổi trạng thái</t>
-        </is>
-      </c>
-      <c r="E70" s="19" t="inlineStr">
-        <is>
-          <t>Phòng ban PB-AUD-01 đang hoạt động</t>
-        </is>
-      </c>
-      <c r="F70" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý phòng ban và chọn Ẩn PB-AUD-01</t>
-        </is>
-      </c>
-      <c r="G70" s="19" t="inlineStr">
-        <is>
-          <t>PB-AUD-01; ACTIVE → INACTIVE → ACTIVE</t>
-        </is>
-      </c>
-      <c r="H70" s="19" t="inlineStr">
-        <is>
-          <t>Mỗi thao tác thành công có một log UPDATE phản ánh đúng thay đổi Trạng thái. Log ẩn ghi Đang hoạt động sang Đã ẩn; log hiện lại ghi Đã ẩn sang Đang hoạt động. Không được ghi action DELETE vì Ẩn không phải Xóa.</t>
-        </is>
-      </c>
-      <c r="I70" s="19" t="n"/>
-      <c r="J70" s="19" t="n"/>
-      <c r="K70" s="19" t="n"/>
-    </row>
-    <row r="71" ht="30" customHeight="1">
-      <c r="A71" s="4" t="n"/>
-      <c r="B71" s="4" t="n"/>
-      <c r="C71" s="4" t="n"/>
-      <c r="D71" s="4" t="n"/>
-      <c r="E71" s="4" t="n"/>
-      <c r="F71" s="19" t="inlineStr">
-        <is>
-          <t>2. Kiểm tra bản ghi chuyển sang Đã ẩn</t>
-        </is>
-      </c>
-      <c r="G71" s="4" t="n"/>
-      <c r="H71" s="4" t="n"/>
-      <c r="I71" s="4" t="n"/>
-      <c r="J71" s="4" t="n"/>
-      <c r="K71" s="4" t="n"/>
-    </row>
-    <row r="72" ht="30" customHeight="1">
-      <c r="A72" s="4" t="n"/>
-      <c r="B72" s="4" t="n"/>
-      <c r="C72" s="4" t="n"/>
-      <c r="D72" s="4" t="n"/>
-      <c r="E72" s="4" t="n"/>
-      <c r="F72" s="19" t="inlineStr">
-        <is>
-          <t>3. Mở Nhật ký và tìm log mới nhất</t>
-        </is>
-      </c>
-      <c r="G72" s="4" t="n"/>
-      <c r="H72" s="4" t="n"/>
-      <c r="I72" s="4" t="n"/>
-      <c r="J72" s="4" t="n"/>
-      <c r="K72" s="4" t="n"/>
-    </row>
-    <row r="73" ht="30" customHeight="1">
-      <c r="A73" s="4" t="n"/>
-      <c r="B73" s="4" t="n"/>
-      <c r="C73" s="4" t="n"/>
-      <c r="D73" s="4" t="n"/>
-      <c r="E73" s="4" t="n"/>
-      <c r="F73" s="19" t="inlineStr">
-        <is>
-          <t>4. Quay lại trang quản lý và chọn Hiện</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="n"/>
-      <c r="H73" s="4" t="n"/>
-      <c r="I73" s="4" t="n"/>
-      <c r="J73" s="4" t="n"/>
-      <c r="K73" s="4" t="n"/>
-    </row>
-    <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="5" t="n"/>
-      <c r="B74" s="5" t="n"/>
-      <c r="C74" s="5" t="n"/>
-      <c r="D74" s="5" t="n"/>
-      <c r="E74" s="5" t="n"/>
-      <c r="F74" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở Nhật ký và đối chiếu log mới nhất lần nữa</t>
-        </is>
-      </c>
-      <c r="G74" s="5" t="n"/>
-      <c r="H74" s="5" t="n"/>
-      <c r="I74" s="5" t="n"/>
-      <c r="J74" s="5" t="n"/>
-      <c r="K74" s="5" t="n"/>
-    </row>
-    <row r="75" ht="30" customHeight="1">
-      <c r="A75" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-4</t>
-        </is>
-      </c>
-      <c r="B75" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Mô hình AI</t>
-        </is>
-      </c>
-      <c r="C75" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-AI-001</t>
-        </is>
-      </c>
-      <c r="D75" s="19" t="inlineStr">
-        <is>
-          <t>Tạo Mô hình AI và xác nhận Nhật ký lưu đúng hành động</t>
-        </is>
-      </c>
-      <c r="E75" s="19" t="inlineStr">
-        <is>
-          <t>Admin đã đăng nhập; chưa có bản ghi mang mã AI-AUD-01</t>
-        </is>
-      </c>
-      <c r="F75" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý mô hình AI</t>
-        </is>
-      </c>
-      <c r="G75" s="19" t="inlineStr">
-        <is>
-          <t>AI-AUD-01; dữ liệu giả hợp lệ</t>
-        </is>
-      </c>
-      <c r="H75" s="19" t="inlineStr">
-        <is>
-          <t>Bản ghi được tạo đúng một lần. Nhật ký có entity AiModelRegistry, action CREATE, đúng ID/mã, Admin và thời gian. Các trường được tạo xuất hiện trong danh sách thay đổi; không hiển thị mật khẩu, khóa bí mật hoặc dữ liệu nhận dạng khuôn mặt.</t>
-        </is>
-      </c>
-      <c r="I75" s="19" t="n"/>
-      <c r="J75" s="19" t="n"/>
-      <c r="K75" s="19" t="n"/>
-    </row>
-    <row r="76" ht="30" customHeight="1">
-      <c r="A76" s="4" t="n"/>
-      <c r="B76" s="4" t="n"/>
-      <c r="C76" s="4" t="n"/>
-      <c r="D76" s="4" t="n"/>
-      <c r="E76" s="4" t="n"/>
-      <c r="F76" s="19" t="inlineStr">
-        <is>
-          <t>2. Chọn thêm mô hình ai, nhập dữ liệu có mã AI-AUD-01 rồi lưu</t>
-        </is>
-      </c>
-      <c r="G76" s="4" t="n"/>
-      <c r="H76" s="4" t="n"/>
-      <c r="I76" s="4" t="n"/>
-      <c r="J76" s="4" t="n"/>
-      <c r="K76" s="4" t="n"/>
-    </row>
-    <row r="77" ht="30" customHeight="1">
-      <c r="A77" s="4" t="n"/>
-      <c r="B77" s="4" t="n"/>
-      <c r="C77" s="4" t="n"/>
-      <c r="D77" s="4" t="n"/>
-      <c r="E77" s="4" t="n"/>
-      <c r="F77" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận bản ghi xuất hiện trong danh sách</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="n"/>
-      <c r="H77" s="4" t="n"/>
-      <c r="I77" s="4" t="n"/>
-      <c r="J77" s="4" t="n"/>
-      <c r="K77" s="4" t="n"/>
-    </row>
-    <row r="78" ht="30" customHeight="1">
-      <c r="A78" s="4" t="n"/>
-      <c r="B78" s="4" t="n"/>
-      <c r="C78" s="4" t="n"/>
-      <c r="D78" s="4" t="n"/>
-      <c r="E78" s="4" t="n"/>
-      <c r="F78" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại thời gian hoàn tất</t>
-        </is>
-      </c>
-      <c r="G78" s="4" t="n"/>
-      <c r="H78" s="4" t="n"/>
-      <c r="I78" s="4" t="n"/>
-      <c r="J78" s="4" t="n"/>
-      <c r="K78" s="4" t="n"/>
-    </row>
-    <row r="79" ht="30" customHeight="1">
-      <c r="A79" s="4" t="n"/>
-      <c r="B79" s="4" t="n"/>
-      <c r="C79" s="4" t="n"/>
-      <c r="D79" s="4" t="n"/>
-      <c r="E79" s="4" t="n"/>
-      <c r="F79" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="n"/>
-      <c r="H79" s="4" t="n"/>
-      <c r="I79" s="4" t="n"/>
-      <c r="J79" s="4" t="n"/>
-      <c r="K79" s="4" t="n"/>
-    </row>
-    <row r="80" ht="30" customHeight="1">
-      <c r="A80" s="4" t="n"/>
-      <c r="B80" s="4" t="n"/>
-      <c r="C80" s="4" t="n"/>
-      <c r="D80" s="4" t="n"/>
-      <c r="E80" s="4" t="n"/>
-      <c r="F80" s="19" t="inlineStr">
-        <is>
-          <t>6. Lọc theo đối tượng Mô hình AI và tìm AI-AUD-01</t>
-        </is>
-      </c>
-      <c r="G80" s="4" t="n"/>
-      <c r="H80" s="4" t="n"/>
-      <c r="I80" s="4" t="n"/>
-      <c r="J80" s="4" t="n"/>
-      <c r="K80" s="4" t="n"/>
-    </row>
-    <row r="81" ht="30" customHeight="1">
-      <c r="A81" s="5" t="n"/>
-      <c r="B81" s="5" t="n"/>
-      <c r="C81" s="5" t="n"/>
-      <c r="D81" s="5" t="n"/>
-      <c r="E81" s="5" t="n"/>
-      <c r="F81" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log mới nhất và đối chiếu thông tin</t>
-        </is>
-      </c>
-      <c r="G81" s="5" t="n"/>
-      <c r="H81" s="5" t="n"/>
-      <c r="I81" s="5" t="n"/>
-      <c r="J81" s="5" t="n"/>
-      <c r="K81" s="5" t="n"/>
-    </row>
-    <row r="82" ht="30" customHeight="1">
-      <c r="A82" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-4</t>
-        </is>
-      </c>
-      <c r="B82" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Mô hình AI</t>
-        </is>
-      </c>
-      <c r="C82" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-AI-002</t>
-        </is>
-      </c>
-      <c r="D82" s="19" t="inlineStr">
-        <is>
-          <t>Sửa một trường của Mô hình AI và kiểm tra giá trị trước/sau trong Nhật ký</t>
-        </is>
-      </c>
-      <c r="E82" s="19" t="inlineStr">
-        <is>
-          <t>Mô hình AI AI-AUD-01 tồn tại; phiên bản hiện là 1.0</t>
-        </is>
-      </c>
-      <c r="F82" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý mô hình AI và chọn AI-AUD-01</t>
-        </is>
-      </c>
-      <c r="G82" s="19" t="inlineStr">
-        <is>
-          <t>phiên bản: 1.0 → 1.1</t>
-        </is>
-      </c>
-      <c r="H82" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký có action UPDATE và chỉ ghi đúng trường phiên bản đã đổi từ 1.0 sang 1.1. Các trường không chỉnh sửa không bị ghi nhầm. Người thực hiện, thời gian và ID đối tượng đúng với thao tác vừa hoàn tất.</t>
-        </is>
-      </c>
-      <c r="I82" s="19" t="n"/>
-      <c r="J82" s="19" t="n"/>
-      <c r="K82" s="19" t="n"/>
-    </row>
-    <row r="83" ht="30" customHeight="1">
-      <c r="A83" s="4" t="n"/>
-      <c r="B83" s="4" t="n"/>
-      <c r="C83" s="4" t="n"/>
-      <c r="D83" s="4" t="n"/>
-      <c r="E83" s="4" t="n"/>
-      <c r="F83" s="19" t="inlineStr">
-        <is>
-          <t>2. Đổi phiên bản từ 1.0 thành 1.1 rồi lưu</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="n"/>
-      <c r="H83" s="4" t="n"/>
-      <c r="I83" s="4" t="n"/>
-      <c r="J83" s="4" t="n"/>
-      <c r="K83" s="4" t="n"/>
-    </row>
-    <row r="84" ht="30" customHeight="1">
-      <c r="A84" s="4" t="n"/>
-      <c r="B84" s="4" t="n"/>
-      <c r="C84" s="4" t="n"/>
-      <c r="D84" s="4" t="n"/>
-      <c r="E84" s="4" t="n"/>
-      <c r="F84" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận màn hình hiển thị giá trị mới</t>
-        </is>
-      </c>
-      <c r="G84" s="4" t="n"/>
-      <c r="H84" s="4" t="n"/>
-      <c r="I84" s="4" t="n"/>
-      <c r="J84" s="4" t="n"/>
-      <c r="K84" s="4" t="n"/>
-    </row>
-    <row r="85" ht="30" customHeight="1">
-      <c r="A85" s="4" t="n"/>
-      <c r="B85" s="4" t="n"/>
-      <c r="C85" s="4" t="n"/>
-      <c r="D85" s="4" t="n"/>
-      <c r="E85" s="4" t="n"/>
-      <c r="F85" s="19" t="inlineStr">
-        <is>
-          <t>4. Mở Nhật ký hệ thống và tìm {key}</t>
-        </is>
-      </c>
-      <c r="G85" s="4" t="n"/>
-      <c r="H85" s="4" t="n"/>
-      <c r="I85" s="4" t="n"/>
-      <c r="J85" s="4" t="n"/>
-      <c r="K85" s="4" t="n"/>
-    </row>
-    <row r="86" ht="30" customHeight="1">
-      <c r="A86" s="4" t="n"/>
-      <c r="B86" s="4" t="n"/>
-      <c r="C86" s="4" t="n"/>
-      <c r="D86" s="4" t="n"/>
-      <c r="E86" s="4" t="n"/>
-      <c r="F86" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở log UPDATE mới nhất</t>
-        </is>
-      </c>
-      <c r="G86" s="4" t="n"/>
-      <c r="H86" s="4" t="n"/>
-      <c r="I86" s="4" t="n"/>
-      <c r="J86" s="4" t="n"/>
-      <c r="K86" s="4" t="n"/>
-    </row>
-    <row r="87" ht="30" customHeight="1">
-      <c r="A87" s="5" t="n"/>
-      <c r="B87" s="5" t="n"/>
-      <c r="C87" s="5" t="n"/>
-      <c r="D87" s="5" t="n"/>
-      <c r="E87" s="5" t="n"/>
-      <c r="F87" s="19" t="inlineStr">
-        <is>
-          <t>6. Đối chiếu trường thay đổi và giá trị trước/sau</t>
-        </is>
-      </c>
-      <c r="G87" s="5" t="n"/>
-      <c r="H87" s="5" t="n"/>
-      <c r="I87" s="5" t="n"/>
-      <c r="J87" s="5" t="n"/>
-      <c r="K87" s="5" t="n"/>
-    </row>
-    <row r="88" ht="30" customHeight="1">
-      <c r="A88" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-E2E-4</t>
-        </is>
-      </c>
-      <c r="B88" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký thao tác Mô hình AI</t>
-        </is>
-      </c>
-      <c r="C88" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-AI-003</t>
-        </is>
-      </c>
-      <c r="D88" s="19" t="inlineStr">
-        <is>
-          <t>Ẩn rồi hiện lại Mô hình AI và kiểm tra hai lần thay đổi trạng thái</t>
-        </is>
-      </c>
-      <c r="E88" s="19" t="inlineStr">
-        <is>
-          <t>Mô hình AI AI-AUD-01 đang hoạt động</t>
-        </is>
-      </c>
-      <c r="F88" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quản lý mô hình AI và chọn Ẩn AI-AUD-01</t>
-        </is>
-      </c>
-      <c r="G88" s="19" t="inlineStr">
-        <is>
-          <t>AI-AUD-01; ACTIVE → INACTIVE → ACTIVE</t>
-        </is>
-      </c>
-      <c r="H88" s="19" t="inlineStr">
-        <is>
-          <t>Mỗi thao tác thành công có một log UPDATE phản ánh đúng thay đổi Trạng thái. Log ẩn ghi Đang hoạt động sang Đã ẩn; log hiện lại ghi Đã ẩn sang Đang hoạt động. Không được ghi action DELETE vì Ẩn không phải Xóa.</t>
-        </is>
-      </c>
-      <c r="I88" s="19" t="n"/>
-      <c r="J88" s="19" t="n"/>
-      <c r="K88" s="19" t="n"/>
-    </row>
-    <row r="89" ht="30" customHeight="1">
-      <c r="A89" s="4" t="n"/>
-      <c r="B89" s="4" t="n"/>
-      <c r="C89" s="4" t="n"/>
-      <c r="D89" s="4" t="n"/>
-      <c r="E89" s="4" t="n"/>
-      <c r="F89" s="19" t="inlineStr">
-        <is>
-          <t>2. Kiểm tra bản ghi chuyển sang Đã ẩn</t>
-        </is>
-      </c>
-      <c r="G89" s="4" t="n"/>
-      <c r="H89" s="4" t="n"/>
-      <c r="I89" s="4" t="n"/>
-      <c r="J89" s="4" t="n"/>
-      <c r="K89" s="4" t="n"/>
-    </row>
-    <row r="90" ht="30" customHeight="1">
-      <c r="A90" s="4" t="n"/>
-      <c r="B90" s="4" t="n"/>
-      <c r="C90" s="4" t="n"/>
-      <c r="D90" s="4" t="n"/>
-      <c r="E90" s="4" t="n"/>
-      <c r="F90" s="19" t="inlineStr">
-        <is>
-          <t>3. Mở Nhật ký và tìm log mới nhất</t>
-        </is>
-      </c>
-      <c r="G90" s="4" t="n"/>
-      <c r="H90" s="4" t="n"/>
-      <c r="I90" s="4" t="n"/>
-      <c r="J90" s="4" t="n"/>
-      <c r="K90" s="4" t="n"/>
-    </row>
-    <row r="91" ht="30" customHeight="1">
-      <c r="A91" s="4" t="n"/>
-      <c r="B91" s="4" t="n"/>
-      <c r="C91" s="4" t="n"/>
-      <c r="D91" s="4" t="n"/>
-      <c r="E91" s="4" t="n"/>
-      <c r="F91" s="19" t="inlineStr">
-        <is>
-          <t>4. Quay lại trang quản lý và chọn Hiện</t>
-        </is>
-      </c>
-      <c r="G91" s="4" t="n"/>
-      <c r="H91" s="4" t="n"/>
-      <c r="I91" s="4" t="n"/>
-      <c r="J91" s="4" t="n"/>
-      <c r="K91" s="4" t="n"/>
-    </row>
-    <row r="92" ht="30" customHeight="1">
-      <c r="A92" s="5" t="n"/>
-      <c r="B92" s="5" t="n"/>
-      <c r="C92" s="5" t="n"/>
-      <c r="D92" s="5" t="n"/>
-      <c r="E92" s="5" t="n"/>
-      <c r="F92" s="19" t="inlineStr">
-        <is>
-          <t>5. Mở Nhật ký và đối chiếu log mới nhất lần nữa</t>
-        </is>
-      </c>
-      <c r="G92" s="5" t="n"/>
-      <c r="H92" s="5" t="n"/>
-      <c r="I92" s="5" t="n"/>
-      <c r="J92" s="5" t="n"/>
-      <c r="K92" s="5" t="n"/>
-    </row>
-    <row r="93" ht="30" customHeight="1">
-      <c r="A93" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-CLIN-1</t>
-        </is>
-      </c>
-      <c r="B93" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký Bệnh nhân</t>
-        </is>
-      </c>
-      <c r="C93" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-PAT-001</t>
-        </is>
-      </c>
-      <c r="D93" s="19" t="inlineStr">
-        <is>
-          <t>Thực hiện tạo hồ sơ bệnh nhân và kiểm tra Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="E93" s="19" t="inlineStr">
-        <is>
-          <t>Có dữ liệu kiểm thử hợp lệ; người dùng đúng vai trò đã đăng nhập</t>
-        </is>
-      </c>
-      <c r="F93" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Tiếp nhận bệnh nhân</t>
-        </is>
-      </c>
-      <c r="G93" s="19" t="inlineStr">
-        <is>
-          <t>PAT-AUD-01; chỉ dùng dữ liệu bệnh nhân giả</t>
-        </is>
-      </c>
-      <c r="H93" s="19" t="inlineStr">
-        <is>
-          <t>Nghiệp vụ hoàn tất đúng một lần và Nhật ký có entity Patient, action CREATE. Log gắn đúng lượt khám/bệnh nhân, đúng người thực hiện và thời gian. Nội dung y tế nhạy cảm chỉ hiển thị khi đúng quyền/xác minh; blockchain chỉ chứa mã kiểm tra, không chứa tên bệnh nhân, CCCD, chẩn đoán, toa thuốc hoặc file.</t>
-        </is>
-      </c>
-      <c r="I93" s="19" t="n"/>
-      <c r="J93" s="19" t="n"/>
-      <c r="K93" s="19" t="n"/>
-    </row>
-    <row r="94" ht="30" customHeight="1">
-      <c r="A94" s="4" t="n"/>
-      <c r="B94" s="4" t="n"/>
-      <c r="C94" s="4" t="n"/>
-      <c r="D94" s="4" t="n"/>
-      <c r="E94" s="4" t="n"/>
-      <c r="F94" s="19" t="inlineStr">
-        <is>
-          <t>2. Thực hiện tạo hồ sơ bệnh nhân cho mã PAT-AUD-01</t>
-        </is>
-      </c>
-      <c r="G94" s="4" t="n"/>
-      <c r="H94" s="4" t="n"/>
-      <c r="I94" s="4" t="n"/>
-      <c r="J94" s="4" t="n"/>
-      <c r="K94" s="4" t="n"/>
-    </row>
-    <row r="95" ht="30" customHeight="1">
-      <c r="A95" s="4" t="n"/>
-      <c r="B95" s="4" t="n"/>
-      <c r="C95" s="4" t="n"/>
-      <c r="D95" s="4" t="n"/>
-      <c r="E95" s="4" t="n"/>
-      <c r="F95" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận nghiệp vụ hoàn tất trên màn hình</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="n"/>
-      <c r="H95" s="4" t="n"/>
-      <c r="I95" s="4" t="n"/>
-      <c r="J95" s="4" t="n"/>
-      <c r="K95" s="4" t="n"/>
-    </row>
-    <row r="96" ht="30" customHeight="1">
-      <c r="A96" s="4" t="n"/>
-      <c r="B96" s="4" t="n"/>
-      <c r="C96" s="4" t="n"/>
-      <c r="D96" s="4" t="n"/>
-      <c r="E96" s="4" t="n"/>
-      <c r="F96" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại người thực hiện và thời gian</t>
-        </is>
-      </c>
-      <c r="G96" s="4" t="n"/>
-      <c r="H96" s="4" t="n"/>
-      <c r="I96" s="4" t="n"/>
-      <c r="J96" s="4" t="n"/>
-      <c r="K96" s="4" t="n"/>
-    </row>
-    <row r="97" ht="30" customHeight="1">
-      <c r="A97" s="4" t="n"/>
-      <c r="B97" s="4" t="n"/>
-      <c r="C97" s="4" t="n"/>
-      <c r="D97" s="4" t="n"/>
-      <c r="E97" s="4" t="n"/>
-      <c r="F97" s="19" t="inlineStr">
-        <is>
-          <t>5. Đăng nhập Admin và mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G97" s="4" t="n"/>
-      <c r="H97" s="4" t="n"/>
-      <c r="I97" s="4" t="n"/>
-      <c r="J97" s="4" t="n"/>
-      <c r="K97" s="4" t="n"/>
-    </row>
-    <row r="98" ht="30" customHeight="1">
-      <c r="A98" s="4" t="n"/>
-      <c r="B98" s="4" t="n"/>
-      <c r="C98" s="4" t="n"/>
-      <c r="D98" s="4" t="n"/>
-      <c r="E98" s="4" t="n"/>
-      <c r="F98" s="19" t="inlineStr">
-        <is>
-          <t>6. Tìm đối tượng Patient liên quan PAT-AUD-01</t>
-        </is>
-      </c>
-      <c r="G98" s="4" t="n"/>
-      <c r="H98" s="4" t="n"/>
-      <c r="I98" s="4" t="n"/>
-      <c r="J98" s="4" t="n"/>
-      <c r="K98" s="4" t="n"/>
-    </row>
-    <row r="99" ht="30" customHeight="1">
-      <c r="A99" s="5" t="n"/>
-      <c r="B99" s="5" t="n"/>
-      <c r="C99" s="5" t="n"/>
-      <c r="D99" s="5" t="n"/>
-      <c r="E99" s="5" t="n"/>
-      <c r="F99" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log và đối chiếu action, người thực hiện, thời gian và trường thay đổi</t>
-        </is>
-      </c>
-      <c r="G99" s="5" t="n"/>
-      <c r="H99" s="5" t="n"/>
-      <c r="I99" s="5" t="n"/>
-      <c r="J99" s="5" t="n"/>
-      <c r="K99" s="5" t="n"/>
-    </row>
-    <row r="100" ht="30" customHeight="1">
-      <c r="A100" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-CLIN-2</t>
-        </is>
-      </c>
-      <c r="B100" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký Lượt khám</t>
-        </is>
-      </c>
-      <c r="C100" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-VIS-001</t>
-        </is>
-      </c>
-      <c r="D100" s="19" t="inlineStr">
-        <is>
-          <t>Thực hiện tạo lượt khám và kiểm tra Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="E100" s="19" t="inlineStr">
-        <is>
-          <t>Có dữ liệu kiểm thử hợp lệ; người dùng đúng vai trò đã đăng nhập</t>
-        </is>
-      </c>
-      <c r="F100" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Tiếp nhận/đặt lịch khám</t>
-        </is>
-      </c>
-      <c r="G100" s="19" t="inlineStr">
-        <is>
-          <t>VIS-AUD-01; chỉ dùng dữ liệu bệnh nhân giả</t>
-        </is>
-      </c>
-      <c r="H100" s="19" t="inlineStr">
-        <is>
-          <t>Nghiệp vụ hoàn tất đúng một lần và Nhật ký có entity Visit, action CREATE. Log gắn đúng lượt khám/bệnh nhân, đúng người thực hiện và thời gian. Nội dung y tế nhạy cảm chỉ hiển thị khi đúng quyền/xác minh; blockchain chỉ chứa mã kiểm tra, không chứa tên bệnh nhân, CCCD, chẩn đoán, toa thuốc hoặc file.</t>
-        </is>
-      </c>
-      <c r="I100" s="19" t="n"/>
-      <c r="J100" s="19" t="n"/>
-      <c r="K100" s="19" t="n"/>
-    </row>
-    <row r="101" ht="30" customHeight="1">
-      <c r="A101" s="4" t="n"/>
-      <c r="B101" s="4" t="n"/>
-      <c r="C101" s="4" t="n"/>
-      <c r="D101" s="4" t="n"/>
-      <c r="E101" s="4" t="n"/>
-      <c r="F101" s="19" t="inlineStr">
-        <is>
-          <t>2. Thực hiện tạo lượt khám cho mã VIS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G101" s="4" t="n"/>
-      <c r="H101" s="4" t="n"/>
-      <c r="I101" s="4" t="n"/>
-      <c r="J101" s="4" t="n"/>
-      <c r="K101" s="4" t="n"/>
-    </row>
-    <row r="102" ht="30" customHeight="1">
-      <c r="A102" s="4" t="n"/>
-      <c r="B102" s="4" t="n"/>
-      <c r="C102" s="4" t="n"/>
-      <c r="D102" s="4" t="n"/>
-      <c r="E102" s="4" t="n"/>
-      <c r="F102" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận nghiệp vụ hoàn tất trên màn hình</t>
-        </is>
-      </c>
-      <c r="G102" s="4" t="n"/>
-      <c r="H102" s="4" t="n"/>
-      <c r="I102" s="4" t="n"/>
-      <c r="J102" s="4" t="n"/>
-      <c r="K102" s="4" t="n"/>
-    </row>
-    <row r="103" ht="30" customHeight="1">
-      <c r="A103" s="4" t="n"/>
-      <c r="B103" s="4" t="n"/>
-      <c r="C103" s="4" t="n"/>
-      <c r="D103" s="4" t="n"/>
-      <c r="E103" s="4" t="n"/>
-      <c r="F103" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại người thực hiện và thời gian</t>
-        </is>
-      </c>
-      <c r="G103" s="4" t="n"/>
-      <c r="H103" s="4" t="n"/>
-      <c r="I103" s="4" t="n"/>
-      <c r="J103" s="4" t="n"/>
-      <c r="K103" s="4" t="n"/>
-    </row>
-    <row r="104" ht="30" customHeight="1">
-      <c r="A104" s="4" t="n"/>
-      <c r="B104" s="4" t="n"/>
-      <c r="C104" s="4" t="n"/>
-      <c r="D104" s="4" t="n"/>
-      <c r="E104" s="4" t="n"/>
-      <c r="F104" s="19" t="inlineStr">
-        <is>
-          <t>5. Đăng nhập Admin và mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G104" s="4" t="n"/>
-      <c r="H104" s="4" t="n"/>
-      <c r="I104" s="4" t="n"/>
-      <c r="J104" s="4" t="n"/>
-      <c r="K104" s="4" t="n"/>
-    </row>
-    <row r="105" ht="30" customHeight="1">
-      <c r="A105" s="4" t="n"/>
-      <c r="B105" s="4" t="n"/>
-      <c r="C105" s="4" t="n"/>
-      <c r="D105" s="4" t="n"/>
-      <c r="E105" s="4" t="n"/>
-      <c r="F105" s="19" t="inlineStr">
-        <is>
-          <t>6. Tìm đối tượng Visit liên quan VIS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G105" s="4" t="n"/>
-      <c r="H105" s="4" t="n"/>
-      <c r="I105" s="4" t="n"/>
-      <c r="J105" s="4" t="n"/>
-      <c r="K105" s="4" t="n"/>
-    </row>
-    <row r="106" ht="30" customHeight="1">
-      <c r="A106" s="5" t="n"/>
-      <c r="B106" s="5" t="n"/>
-      <c r="C106" s="5" t="n"/>
-      <c r="D106" s="5" t="n"/>
-      <c r="E106" s="5" t="n"/>
-      <c r="F106" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log và đối chiếu action, người thực hiện, thời gian và trường thay đổi</t>
-        </is>
-      </c>
-      <c r="G106" s="5" t="n"/>
-      <c r="H106" s="5" t="n"/>
-      <c r="I106" s="5" t="n"/>
-      <c r="J106" s="5" t="n"/>
-      <c r="K106" s="5" t="n"/>
-    </row>
-    <row r="107" ht="30" customHeight="1">
-      <c r="A107" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-CLIN-3</t>
-        </is>
-      </c>
-      <c r="B107" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký Trạng thái lượt khám</t>
-        </is>
-      </c>
-      <c r="C107" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-VST-001</t>
-        </is>
-      </c>
-      <c r="D107" s="19" t="inlineStr">
-        <is>
-          <t>Thực hiện bắt đầu khám hoặc chuyển trạng thái và kiểm tra Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="E107" s="19" t="inlineStr">
-        <is>
-          <t>Có dữ liệu kiểm thử hợp lệ; người dùng đúng vai trò đã đăng nhập</t>
-        </is>
-      </c>
-      <c r="F107" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Hàng đợi khám bệnh</t>
-        </is>
-      </c>
-      <c r="G107" s="19" t="inlineStr">
-        <is>
-          <t>VIS-AUD-01; chỉ dùng dữ liệu bệnh nhân giả</t>
-        </is>
-      </c>
-      <c r="H107" s="19" t="inlineStr">
-        <is>
-          <t>Nghiệp vụ hoàn tất đúng một lần và Nhật ký có entity Visit, action UPDATE. Log gắn đúng lượt khám/bệnh nhân, đúng người thực hiện và thời gian. Nội dung y tế nhạy cảm chỉ hiển thị khi đúng quyền/xác minh; blockchain chỉ chứa mã kiểm tra, không chứa tên bệnh nhân, CCCD, chẩn đoán, toa thuốc hoặc file.</t>
-        </is>
-      </c>
-      <c r="I107" s="19" t="n"/>
-      <c r="J107" s="19" t="n"/>
-      <c r="K107" s="19" t="n"/>
-    </row>
-    <row r="108" ht="30" customHeight="1">
-      <c r="A108" s="4" t="n"/>
-      <c r="B108" s="4" t="n"/>
-      <c r="C108" s="4" t="n"/>
-      <c r="D108" s="4" t="n"/>
-      <c r="E108" s="4" t="n"/>
-      <c r="F108" s="19" t="inlineStr">
-        <is>
-          <t>2. Thực hiện bắt đầu khám hoặc chuyển trạng thái cho mã VIS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G108" s="4" t="n"/>
-      <c r="H108" s="4" t="n"/>
-      <c r="I108" s="4" t="n"/>
-      <c r="J108" s="4" t="n"/>
-      <c r="K108" s="4" t="n"/>
-    </row>
-    <row r="109" ht="30" customHeight="1">
-      <c r="A109" s="4" t="n"/>
-      <c r="B109" s="4" t="n"/>
-      <c r="C109" s="4" t="n"/>
-      <c r="D109" s="4" t="n"/>
-      <c r="E109" s="4" t="n"/>
-      <c r="F109" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận nghiệp vụ hoàn tất trên màn hình</t>
-        </is>
-      </c>
-      <c r="G109" s="4" t="n"/>
-      <c r="H109" s="4" t="n"/>
-      <c r="I109" s="4" t="n"/>
-      <c r="J109" s="4" t="n"/>
-      <c r="K109" s="4" t="n"/>
-    </row>
-    <row r="110" ht="30" customHeight="1">
-      <c r="A110" s="4" t="n"/>
-      <c r="B110" s="4" t="n"/>
-      <c r="C110" s="4" t="n"/>
-      <c r="D110" s="4" t="n"/>
-      <c r="E110" s="4" t="n"/>
-      <c r="F110" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại người thực hiện và thời gian</t>
-        </is>
-      </c>
-      <c r="G110" s="4" t="n"/>
-      <c r="H110" s="4" t="n"/>
-      <c r="I110" s="4" t="n"/>
-      <c r="J110" s="4" t="n"/>
-      <c r="K110" s="4" t="n"/>
-    </row>
-    <row r="111" ht="30" customHeight="1">
-      <c r="A111" s="4" t="n"/>
-      <c r="B111" s="4" t="n"/>
-      <c r="C111" s="4" t="n"/>
-      <c r="D111" s="4" t="n"/>
-      <c r="E111" s="4" t="n"/>
-      <c r="F111" s="19" t="inlineStr">
-        <is>
-          <t>5. Đăng nhập Admin và mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G111" s="4" t="n"/>
-      <c r="H111" s="4" t="n"/>
-      <c r="I111" s="4" t="n"/>
-      <c r="J111" s="4" t="n"/>
-      <c r="K111" s="4" t="n"/>
-    </row>
-    <row r="112" ht="30" customHeight="1">
-      <c r="A112" s="4" t="n"/>
-      <c r="B112" s="4" t="n"/>
-      <c r="C112" s="4" t="n"/>
-      <c r="D112" s="4" t="n"/>
-      <c r="E112" s="4" t="n"/>
-      <c r="F112" s="19" t="inlineStr">
-        <is>
-          <t>6. Tìm đối tượng Visit liên quan VIS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G112" s="4" t="n"/>
-      <c r="H112" s="4" t="n"/>
-      <c r="I112" s="4" t="n"/>
-      <c r="J112" s="4" t="n"/>
-      <c r="K112" s="4" t="n"/>
-    </row>
-    <row r="113" ht="30" customHeight="1">
-      <c r="A113" s="5" t="n"/>
-      <c r="B113" s="5" t="n"/>
-      <c r="C113" s="5" t="n"/>
-      <c r="D113" s="5" t="n"/>
-      <c r="E113" s="5" t="n"/>
-      <c r="F113" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log và đối chiếu action, người thực hiện, thời gian và trường thay đổi</t>
-        </is>
-      </c>
-      <c r="G113" s="5" t="n"/>
-      <c r="H113" s="5" t="n"/>
-      <c r="I113" s="5" t="n"/>
-      <c r="J113" s="5" t="n"/>
-      <c r="K113" s="5" t="n"/>
-    </row>
-    <row r="114" ht="30" customHeight="1">
-      <c r="A114" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-CLIN-4</t>
-        </is>
-      </c>
-      <c r="B114" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký Kết quả cận lâm sàng</t>
-        </is>
-      </c>
-      <c r="C114" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-RES-001</t>
-        </is>
-      </c>
-      <c r="D114" s="19" t="inlineStr">
-        <is>
-          <t>Thực hiện trả kết quả và kiểm tra Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="E114" s="19" t="inlineStr">
-        <is>
-          <t>Có dữ liệu kiểm thử hợp lệ; người dùng đúng vai trò đã đăng nhập</t>
-        </is>
-      </c>
-      <c r="F114" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Trả kết quả cận lâm sàng</t>
-        </is>
-      </c>
-      <c r="G114" s="19" t="inlineStr">
-        <is>
-          <t>KQ-AUD-01; chỉ dùng dữ liệu bệnh nhân giả</t>
-        </is>
-      </c>
-      <c r="H114" s="19" t="inlineStr">
-        <is>
-          <t>Nghiệp vụ hoàn tất đúng một lần và Nhật ký có entity MedicalResult, action CREATE. Log gắn đúng lượt khám/bệnh nhân, đúng người thực hiện và thời gian. Nội dung y tế nhạy cảm chỉ hiển thị khi đúng quyền/xác minh; blockchain chỉ chứa mã kiểm tra, không chứa tên bệnh nhân, CCCD, chẩn đoán, toa thuốc hoặc file.</t>
-        </is>
-      </c>
-      <c r="I114" s="19" t="n"/>
-      <c r="J114" s="19" t="n"/>
-      <c r="K114" s="19" t="n"/>
-    </row>
-    <row r="115" ht="30" customHeight="1">
-      <c r="A115" s="4" t="n"/>
-      <c r="B115" s="4" t="n"/>
-      <c r="C115" s="4" t="n"/>
-      <c r="D115" s="4" t="n"/>
-      <c r="E115" s="4" t="n"/>
-      <c r="F115" s="19" t="inlineStr">
-        <is>
-          <t>2. Thực hiện trả kết quả cho mã KQ-AUD-01</t>
-        </is>
-      </c>
-      <c r="G115" s="4" t="n"/>
-      <c r="H115" s="4" t="n"/>
-      <c r="I115" s="4" t="n"/>
-      <c r="J115" s="4" t="n"/>
-      <c r="K115" s="4" t="n"/>
-    </row>
-    <row r="116" ht="30" customHeight="1">
-      <c r="A116" s="4" t="n"/>
-      <c r="B116" s="4" t="n"/>
-      <c r="C116" s="4" t="n"/>
-      <c r="D116" s="4" t="n"/>
-      <c r="E116" s="4" t="n"/>
-      <c r="F116" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận nghiệp vụ hoàn tất trên màn hình</t>
-        </is>
-      </c>
-      <c r="G116" s="4" t="n"/>
-      <c r="H116" s="4" t="n"/>
-      <c r="I116" s="4" t="n"/>
-      <c r="J116" s="4" t="n"/>
-      <c r="K116" s="4" t="n"/>
-    </row>
-    <row r="117" ht="30" customHeight="1">
-      <c r="A117" s="4" t="n"/>
-      <c r="B117" s="4" t="n"/>
-      <c r="C117" s="4" t="n"/>
-      <c r="D117" s="4" t="n"/>
-      <c r="E117" s="4" t="n"/>
-      <c r="F117" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại người thực hiện và thời gian</t>
-        </is>
-      </c>
-      <c r="G117" s="4" t="n"/>
-      <c r="H117" s="4" t="n"/>
-      <c r="I117" s="4" t="n"/>
-      <c r="J117" s="4" t="n"/>
-      <c r="K117" s="4" t="n"/>
-    </row>
-    <row r="118" ht="30" customHeight="1">
-      <c r="A118" s="4" t="n"/>
-      <c r="B118" s="4" t="n"/>
-      <c r="C118" s="4" t="n"/>
-      <c r="D118" s="4" t="n"/>
-      <c r="E118" s="4" t="n"/>
-      <c r="F118" s="19" t="inlineStr">
-        <is>
-          <t>5. Đăng nhập Admin và mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G118" s="4" t="n"/>
-      <c r="H118" s="4" t="n"/>
-      <c r="I118" s="4" t="n"/>
-      <c r="J118" s="4" t="n"/>
-      <c r="K118" s="4" t="n"/>
-    </row>
-    <row r="119" ht="30" customHeight="1">
-      <c r="A119" s="4" t="n"/>
-      <c r="B119" s="4" t="n"/>
-      <c r="C119" s="4" t="n"/>
-      <c r="D119" s="4" t="n"/>
-      <c r="E119" s="4" t="n"/>
-      <c r="F119" s="19" t="inlineStr">
-        <is>
-          <t>6. Tìm đối tượng MedicalResult liên quan KQ-AUD-01</t>
-        </is>
-      </c>
-      <c r="G119" s="4" t="n"/>
-      <c r="H119" s="4" t="n"/>
-      <c r="I119" s="4" t="n"/>
-      <c r="J119" s="4" t="n"/>
-      <c r="K119" s="4" t="n"/>
-    </row>
-    <row r="120" ht="30" customHeight="1">
-      <c r="A120" s="5" t="n"/>
-      <c r="B120" s="5" t="n"/>
-      <c r="C120" s="5" t="n"/>
-      <c r="D120" s="5" t="n"/>
-      <c r="E120" s="5" t="n"/>
-      <c r="F120" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log và đối chiếu action, người thực hiện, thời gian và trường thay đổi</t>
-        </is>
-      </c>
-      <c r="G120" s="5" t="n"/>
-      <c r="H120" s="5" t="n"/>
-      <c r="I120" s="5" t="n"/>
-      <c r="J120" s="5" t="n"/>
-      <c r="K120" s="5" t="n"/>
-    </row>
-    <row r="121" ht="30" customHeight="1">
-      <c r="A121" s="19" t="inlineStr">
-        <is>
-          <t>S-AUD-CLIN-5</t>
-        </is>
-      </c>
-      <c r="B121" s="19" t="inlineStr">
-        <is>
-          <t>Nhật ký Kết luận khám</t>
-        </is>
-      </c>
-      <c r="C121" s="19" t="inlineStr">
-        <is>
-          <t>TC-AUD-CON-001</t>
-        </is>
-      </c>
-      <c r="D121" s="19" t="inlineStr">
-        <is>
-          <t>Thực hiện lưu kết luận cuối và kiểm tra Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="E121" s="19" t="inlineStr">
-        <is>
-          <t>Có dữ liệu kiểm thử hợp lệ; người dùng đúng vai trò đã đăng nhập</t>
-        </is>
-      </c>
-      <c r="F121" s="19" t="inlineStr">
-        <is>
-          <t>1. Mở Quy trình khám của bác sĩ</t>
-        </is>
-      </c>
-      <c r="G121" s="19" t="inlineStr">
-        <is>
-          <t>VIS-AUD-01; chỉ dùng dữ liệu bệnh nhân giả</t>
-        </is>
-      </c>
-      <c r="H121" s="19" t="inlineStr">
-        <is>
-          <t>Nghiệp vụ hoàn tất đúng một lần và Nhật ký có entity MedicalConclusion, action CREATE/UPDATE theo việc đã có kết luận hay chưa. Log gắn đúng lượt khám/bệnh nhân, đúng người thực hiện và thời gian. Nội dung y tế nhạy cảm chỉ hiển thị khi đúng quyền/xác minh; blockchain chỉ chứa mã kiểm tra, không chứa tên bệnh nhân, CCCD, chẩn đoán, toa thuốc hoặc file.</t>
-        </is>
-      </c>
-      <c r="I121" s="19" t="n"/>
-      <c r="J121" s="19" t="n"/>
-      <c r="K121" s="19" t="n"/>
-    </row>
-    <row r="122" ht="30" customHeight="1">
-      <c r="A122" s="4" t="n"/>
-      <c r="B122" s="4" t="n"/>
-      <c r="C122" s="4" t="n"/>
-      <c r="D122" s="4" t="n"/>
-      <c r="E122" s="4" t="n"/>
-      <c r="F122" s="19" t="inlineStr">
-        <is>
-          <t>2. Thực hiện lưu kết luận cuối cho mã VIS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G122" s="4" t="n"/>
-      <c r="H122" s="4" t="n"/>
-      <c r="I122" s="4" t="n"/>
-      <c r="J122" s="4" t="n"/>
-      <c r="K122" s="4" t="n"/>
-    </row>
-    <row r="123" ht="30" customHeight="1">
-      <c r="A123" s="4" t="n"/>
-      <c r="B123" s="4" t="n"/>
-      <c r="C123" s="4" t="n"/>
-      <c r="D123" s="4" t="n"/>
-      <c r="E123" s="4" t="n"/>
-      <c r="F123" s="19" t="inlineStr">
-        <is>
-          <t>3. Xác nhận nghiệp vụ hoàn tất trên màn hình</t>
-        </is>
-      </c>
-      <c r="G123" s="4" t="n"/>
-      <c r="H123" s="4" t="n"/>
-      <c r="I123" s="4" t="n"/>
-      <c r="J123" s="4" t="n"/>
-      <c r="K123" s="4" t="n"/>
-    </row>
-    <row r="124" ht="30" customHeight="1">
-      <c r="A124" s="4" t="n"/>
-      <c r="B124" s="4" t="n"/>
-      <c r="C124" s="4" t="n"/>
-      <c r="D124" s="4" t="n"/>
-      <c r="E124" s="4" t="n"/>
-      <c r="F124" s="19" t="inlineStr">
-        <is>
-          <t>4. Ghi lại người thực hiện và thời gian</t>
-        </is>
-      </c>
-      <c r="G124" s="4" t="n"/>
-      <c r="H124" s="4" t="n"/>
-      <c r="I124" s="4" t="n"/>
-      <c r="J124" s="4" t="n"/>
-      <c r="K124" s="4" t="n"/>
-    </row>
-    <row r="125" ht="30" customHeight="1">
-      <c r="A125" s="4" t="n"/>
-      <c r="B125" s="4" t="n"/>
-      <c r="C125" s="4" t="n"/>
-      <c r="D125" s="4" t="n"/>
-      <c r="E125" s="4" t="n"/>
-      <c r="F125" s="19" t="inlineStr">
-        <is>
-          <t>5. Đăng nhập Admin và mở Nhật ký hệ thống</t>
-        </is>
-      </c>
-      <c r="G125" s="4" t="n"/>
-      <c r="H125" s="4" t="n"/>
-      <c r="I125" s="4" t="n"/>
-      <c r="J125" s="4" t="n"/>
-      <c r="K125" s="4" t="n"/>
-    </row>
-    <row r="126" ht="30" customHeight="1">
-      <c r="A126" s="4" t="n"/>
-      <c r="B126" s="4" t="n"/>
-      <c r="C126" s="4" t="n"/>
-      <c r="D126" s="4" t="n"/>
-      <c r="E126" s="4" t="n"/>
-      <c r="F126" s="19" t="inlineStr">
-        <is>
-          <t>6. Tìm đối tượng MedicalConclusion liên quan VIS-AUD-01</t>
-        </is>
-      </c>
-      <c r="G126" s="4" t="n"/>
-      <c r="H126" s="4" t="n"/>
-      <c r="I126" s="4" t="n"/>
-      <c r="J126" s="4" t="n"/>
-      <c r="K126" s="4" t="n"/>
-    </row>
-    <row r="127" ht="30" customHeight="1">
-      <c r="A127" s="5" t="n"/>
-      <c r="B127" s="5" t="n"/>
-      <c r="C127" s="5" t="n"/>
-      <c r="D127" s="5" t="n"/>
-      <c r="E127" s="5" t="n"/>
-      <c r="F127" s="19" t="inlineStr">
-        <is>
-          <t>7. Mở log và đối chiếu action, người thực hiện, thời gian và trường thay đổi</t>
-        </is>
-      </c>
-      <c r="G127" s="5" t="n"/>
-      <c r="H127" s="5" t="n"/>
-      <c r="I127" s="5" t="n"/>
-      <c r="J127" s="5" t="n"/>
-      <c r="K127" s="5" t="n"/>
+          <t xml:space="preserve">Bước 1: Chuẩn bị một audit batch có trạng thái artifact ready.
+Bước 2: Giả lập blockchain hoặc mạng không phản hồi khi commit checkpoint.
+Bước 3: Kiểm tra batch giữ trạng thái chờ retry.
+Bước 4: Khôi phục kết nối blockchain.
+Bước 5: Chạy lại quy trình anchor và kiểm tra artifactUri, artifactHash và checkpoint.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Batch trạng thái ARTIFACT_READY; lỗi là blockchain network outage tạm thời</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hệ thống giữ nguyên artifactUri và artifactHash, retry commit checkpoint khi kết nối phục hồi, chuyển batch sang trạng thái đã anchor và không tạo artifact hoặc batch mới trùng.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đạt. Batch chờ retry được anchor thành công sau khi blockchain hoạt động lại.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Passed</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package: Audit logs và blockchain</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H127"/>
-  <mergeCells count="175">
-    <mergeCell ref="B57:B63"/>
-    <mergeCell ref="B88:B92"/>
-    <mergeCell ref="D57:D63"/>
+  <autoFilter ref="A1:K15"/>
+  <mergeCells count="12">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="A12:A13"/>
     <mergeCell ref="B12:B13"/>
-    <mergeCell ref="H82:H87"/>
-    <mergeCell ref="C21:C27"/>
-    <mergeCell ref="B107:B113"/>
-    <mergeCell ref="H100:H106"/>
-    <mergeCell ref="D107:D113"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D121:D127"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="H57:H63"/>
+    <mergeCell ref="A14:A15"/>
     <mergeCell ref="B14:B15"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="C70:C74"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="C64:C69"/>
-    <mergeCell ref="E64:E69"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="D93:D99"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="E46:E51"/>
-    <mergeCell ref="E18:E20"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="A114:A120"/>
-    <mergeCell ref="E21:E27"/>
-    <mergeCell ref="A46:A51"/>
-    <mergeCell ref="G64:G69"/>
-    <mergeCell ref="B21:B27"/>
-    <mergeCell ref="D21:D27"/>
-    <mergeCell ref="H28:H33"/>
-    <mergeCell ref="B100:B106"/>
-    <mergeCell ref="D100:D106"/>
-    <mergeCell ref="C88:C92"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E88:E92"/>
-    <mergeCell ref="G57:G63"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C82:C87"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E107:E113"/>
-    <mergeCell ref="H21:H27"/>
-    <mergeCell ref="G107:G113"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="D70:D74"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="B39:B45"/>
-    <mergeCell ref="H114:H120"/>
-    <mergeCell ref="E34:E38"/>
-    <mergeCell ref="H88:H92"/>
-    <mergeCell ref="G34:G38"/>
-    <mergeCell ref="C52:C56"/>
-    <mergeCell ref="H7:H9"/>
-    <mergeCell ref="G93:G99"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="G4:G6"/>
-    <mergeCell ref="H18:H20"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="E75:E81"/>
-    <mergeCell ref="A100:A106"/>
-    <mergeCell ref="G75:G81"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="B82:B87"/>
-    <mergeCell ref="C46:C51"/>
-    <mergeCell ref="E100:E106"/>
-    <mergeCell ref="G100:G106"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="D34:D38"/>
-    <mergeCell ref="H107:H113"/>
-    <mergeCell ref="B28:B33"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="D28:D33"/>
-    <mergeCell ref="G70:G74"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="A70:A74"/>
-    <mergeCell ref="E39:E45"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="H34:H38"/>
-    <mergeCell ref="G39:G45"/>
-    <mergeCell ref="H52:H56"/>
-    <mergeCell ref="C121:C127"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="B93:B99"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="H39:H45"/>
-    <mergeCell ref="E114:E120"/>
-    <mergeCell ref="C93:C99"/>
-    <mergeCell ref="G121:G127"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B46:B51"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D46:D51"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="H75:H81"/>
-    <mergeCell ref="C57:C63"/>
-    <mergeCell ref="E57:E63"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="H64:H69"/>
-    <mergeCell ref="E28:E33"/>
-    <mergeCell ref="G28:G33"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B114:B120"/>
-    <mergeCell ref="A93:A99"/>
-    <mergeCell ref="A34:A38"/>
-    <mergeCell ref="D88:D92"/>
-    <mergeCell ref="D114:D120"/>
-    <mergeCell ref="C34:C38"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="A88:A92"/>
-    <mergeCell ref="G21:G27"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="E93:E99"/>
-    <mergeCell ref="H121:H127"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="A39:A45"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="D52:D56"/>
-    <mergeCell ref="C75:C81"/>
-    <mergeCell ref="H93:H99"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="G46:G51"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="A75:A81"/>
-    <mergeCell ref="C100:C106"/>
-    <mergeCell ref="D75:D81"/>
-    <mergeCell ref="C114:C120"/>
-    <mergeCell ref="A64:A69"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="A82:A87"/>
-    <mergeCell ref="A21:A27"/>
-    <mergeCell ref="E70:E74"/>
-    <mergeCell ref="G114:G120"/>
-    <mergeCell ref="A57:A63"/>
-    <mergeCell ref="C39:C45"/>
-    <mergeCell ref="G88:G92"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="E82:E87"/>
-    <mergeCell ref="G82:G87"/>
-    <mergeCell ref="A52:A56"/>
-    <mergeCell ref="A121:A127"/>
-    <mergeCell ref="H46:H51"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="D39:D45"/>
-    <mergeCell ref="H4:H6"/>
-    <mergeCell ref="E52:E56"/>
-    <mergeCell ref="G52:G56"/>
-    <mergeCell ref="E121:E127"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="A107:A113"/>
-    <mergeCell ref="C107:C113"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="B64:B69"/>
-    <mergeCell ref="D64:D69"/>
-    <mergeCell ref="B121:B127"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="D82:D87"/>
-    <mergeCell ref="C28:C33"/>
-    <mergeCell ref="H70:H74"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -7876,7 +5734,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -8257,7 +6115,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
@@ -15389,7 +13247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -16131,7 +13989,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -17098,7 +14956,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -26486,7 +24344,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
@@ -30868,7 +28726,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -33352,7 +31210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
@@ -36108,7 +33966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>

</xml_diff>